<commit_message>
Replace forecast CSVs with interval-based versions
Deleted individual disease forecast CSVs and added new forecast files with intervals under 'Forecasts_with_intervals'. Updated related appendix images and model results to reflect the new forecast data structure.
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Best_model_outcome.xlsx
+++ b/Outcome/Appendix/Best_model_outcome.xlsx
@@ -44,25 +44,25 @@
     <t xml:space="preserve">Pneumonia</t>
   </si>
   <si>
-    <t xml:space="preserve">TBATS</t>
+    <t xml:space="preserve">ETS</t>
   </si>
   <si>
     <t xml:space="preserve">Respiratory IDs</t>
   </si>
   <si>
+    <t xml:space="preserve">Neural Network</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBATS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SARIMA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bayesian structural</t>
   </si>
   <si>
-    <t xml:space="preserve">Neural Network</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ETS</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hybrid**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SARIMA</t>
   </si>
   <si>
     <t xml:space="preserve">Influenza</t>
@@ -506,22 +506,22 @@
         <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>11.59</v>
+        <v>13.78</v>
       </c>
       <c r="D2" t="n">
-        <v>3760.98</v>
+        <v>4515.34</v>
       </c>
       <c r="E2" t="n">
-        <v>0.75</v>
+        <v>0.86</v>
       </c>
       <c r="F2" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.75</v>
+        <v>-0.86</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="s">
         <v>11</v>
@@ -535,19 +535,19 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>11.86</v>
+        <v>17.65</v>
       </c>
       <c r="D3" t="n">
-        <v>4119.05</v>
+        <v>5427.33</v>
       </c>
       <c r="E3" t="n">
-        <v>0.75</v>
+        <v>1.15</v>
       </c>
       <c r="F3" t="n">
-        <v>0.57</v>
+        <v>0.19</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.75</v>
+        <v>-1.15</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -564,22 +564,22 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>16.84</v>
+        <v>11.59</v>
       </c>
       <c r="D4" t="n">
-        <v>5100.87</v>
+        <v>3760.98</v>
       </c>
       <c r="E4" t="n">
-        <v>1.15</v>
+        <v>0.75</v>
       </c>
       <c r="F4" t="n">
-        <v>0.24</v>
+        <v>0.57</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.15</v>
+        <v>-0.75</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="s">
         <v>11</v>
@@ -593,19 +593,19 @@
         <v>14</v>
       </c>
       <c r="C5" t="n">
-        <v>13.78</v>
+        <v>17.64</v>
       </c>
       <c r="D5" t="n">
-        <v>4515.34</v>
+        <v>5826.04</v>
       </c>
       <c r="E5" t="n">
-        <v>0.86</v>
+        <v>1.18</v>
       </c>
       <c r="F5" t="n">
-        <v>0.59</v>
+        <v>0.34</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.86</v>
+        <v>-1.18</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -622,19 +622,19 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>14.2</v>
+        <v>11.86</v>
       </c>
       <c r="D6" t="n">
-        <v>4668.78</v>
+        <v>4119.05</v>
       </c>
       <c r="E6" t="n">
-        <v>0.95</v>
+        <v>0.75</v>
       </c>
       <c r="F6" t="n">
-        <v>0.46</v>
+        <v>0.57</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.95</v>
+        <v>-0.75</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -651,19 +651,19 @@
         <v>16</v>
       </c>
       <c r="C7" t="n">
-        <v>17.64</v>
+        <v>14.5</v>
       </c>
       <c r="D7" t="n">
-        <v>5826.04</v>
+        <v>4803.29</v>
       </c>
       <c r="E7" t="n">
-        <v>1.18</v>
+        <v>0.97</v>
       </c>
       <c r="F7" t="n">
-        <v>0.34</v>
+        <v>0.44</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.18</v>
+        <v>-0.97</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -677,22 +677,22 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C8" t="n">
-        <v>101.28</v>
+        <v>56.88</v>
       </c>
       <c r="D8" t="n">
-        <v>25326.8</v>
+        <v>16863.01</v>
       </c>
       <c r="E8" t="n">
-        <v>18.85</v>
+        <v>2.4</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5</v>
+        <v>0.36</v>
       </c>
       <c r="G8" t="n">
-        <v>-18.85</v>
+        <v>-2.4</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -706,22 +706,22 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>56.16</v>
+        <v>103.34</v>
       </c>
       <c r="D9" t="n">
-        <v>16814.32</v>
+        <v>25636.96</v>
       </c>
       <c r="E9" t="n">
-        <v>2.36</v>
+        <v>19.1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.33</v>
+        <v>0.46</v>
       </c>
       <c r="G9" t="n">
-        <v>-2.36</v>
+        <v>-19.1</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -735,7 +735,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C10" t="n">
         <v>119.84</v>
@@ -767,22 +767,22 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>55.67</v>
+        <v>46.61</v>
       </c>
       <c r="D11" t="n">
-        <v>15505.1</v>
+        <v>17747.28</v>
       </c>
       <c r="E11" t="n">
-        <v>1.81</v>
+        <v>1.17</v>
       </c>
       <c r="F11" t="n">
-        <v>0.47</v>
+        <v>0.18</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.81</v>
+        <v>-1.17</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" t="s">
         <v>11</v>
@@ -796,22 +796,22 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>46.61</v>
+        <v>51.69</v>
       </c>
       <c r="D12" t="n">
-        <v>17747.28</v>
+        <v>16621.43</v>
       </c>
       <c r="E12" t="n">
-        <v>1.17</v>
+        <v>2.38</v>
       </c>
       <c r="F12" t="n">
-        <v>0.18</v>
+        <v>0.26</v>
       </c>
       <c r="G12" t="n">
-        <v>-1.17</v>
+        <v>-2.38</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" t="s">
         <v>11</v>
@@ -822,22 +822,22 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>51.69</v>
+        <v>55.67</v>
       </c>
       <c r="D13" t="n">
-        <v>16621.43</v>
+        <v>15505.1</v>
       </c>
       <c r="E13" t="n">
-        <v>2.38</v>
+        <v>1.81</v>
       </c>
       <c r="F13" t="n">
-        <v>0.26</v>
+        <v>0.47</v>
       </c>
       <c r="G13" t="n">
-        <v>-2.38</v>
+        <v>-1.81</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -851,25 +851,25 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>25.44</v>
+        <v>19.2</v>
       </c>
       <c r="D14" t="n">
-        <v>2234.67</v>
+        <v>1316.98</v>
       </c>
       <c r="E14" t="n">
-        <v>1.2</v>
+        <v>0.92</v>
       </c>
       <c r="F14" t="n">
-        <v>0.97</v>
+        <v>0.94</v>
       </c>
       <c r="G14" t="n">
-        <v>-1.2</v>
+        <v>-0.92</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="s">
         <v>11</v>
@@ -880,22 +880,22 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C15" t="n">
-        <v>37.15</v>
+        <v>27.16</v>
       </c>
       <c r="D15" t="n">
-        <v>3190.05</v>
+        <v>2493.27</v>
       </c>
       <c r="E15" t="n">
-        <v>1.45</v>
+        <v>1.23</v>
       </c>
       <c r="F15" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="G15" t="n">
-        <v>-1.45</v>
+        <v>-1.23</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -909,7 +909,7 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C16" t="n">
         <v>30.49</v>
@@ -941,19 +941,19 @@
         <v>14</v>
       </c>
       <c r="C17" t="n">
-        <v>33.53</v>
+        <v>21.95</v>
       </c>
       <c r="D17" t="n">
-        <v>3256.09</v>
+        <v>2067.97</v>
       </c>
       <c r="E17" t="n">
-        <v>1.37</v>
+        <v>1.08</v>
       </c>
       <c r="F17" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.37</v>
+        <v>-1.08</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -967,22 +967,22 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C18" t="n">
-        <v>21.29</v>
+        <v>37.15</v>
       </c>
       <c r="D18" t="n">
-        <v>1201.94</v>
+        <v>3190.05</v>
       </c>
       <c r="E18" t="n">
-        <v>1.13</v>
+        <v>1.45</v>
       </c>
       <c r="F18" t="n">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="G18" t="n">
-        <v>-1.13</v>
+        <v>-1.45</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -996,25 +996,25 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C19" t="n">
-        <v>21.95</v>
+        <v>33.53</v>
       </c>
       <c r="D19" t="n">
-        <v>2067.97</v>
+        <v>3256.09</v>
       </c>
       <c r="E19" t="n">
-        <v>1.08</v>
+        <v>1.37</v>
       </c>
       <c r="F19" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="G19" t="n">
-        <v>-1.08</v>
+        <v>-1.37</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" t="s">
         <v>11</v>
@@ -1025,22 +1025,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" t="n">
-        <v>20.01</v>
+        <v>33.51</v>
       </c>
       <c r="D20" t="n">
-        <v>49.74</v>
+        <v>71.07</v>
       </c>
       <c r="E20" t="n">
-        <v>2.92</v>
+        <v>4.66</v>
       </c>
       <c r="F20" t="n">
-        <v>0.47</v>
+        <v>0.29</v>
       </c>
       <c r="G20" t="n">
-        <v>-2.92</v>
+        <v>-4.66</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1054,25 +1054,25 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C21" t="n">
-        <v>22.78</v>
+        <v>20.01</v>
       </c>
       <c r="D21" t="n">
-        <v>52.43</v>
+        <v>49.74</v>
       </c>
       <c r="E21" t="n">
-        <v>2.74</v>
+        <v>2.92</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6</v>
+        <v>0.47</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.74</v>
+        <v>-2.92</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" t="s">
         <v>11</v>
@@ -1083,22 +1083,22 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C22" t="n">
-        <v>24.48</v>
+        <v>22.11</v>
       </c>
       <c r="D22" t="n">
-        <v>56.77</v>
+        <v>53.28</v>
       </c>
       <c r="E22" t="n">
-        <v>4.96</v>
+        <v>3.84</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7</v>
+        <v>0.58</v>
       </c>
       <c r="G22" t="n">
-        <v>-4.96</v>
+        <v>-3.84</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1115,19 +1115,19 @@
         <v>12</v>
       </c>
       <c r="C23" t="n">
-        <v>33.51</v>
+        <v>25.05</v>
       </c>
       <c r="D23" t="n">
-        <v>71.07</v>
+        <v>58.07</v>
       </c>
       <c r="E23" t="n">
-        <v>4.66</v>
+        <v>5.47</v>
       </c>
       <c r="F23" t="n">
-        <v>0.29</v>
+        <v>0.69</v>
       </c>
       <c r="G23" t="n">
-        <v>-4.66</v>
+        <v>-5.47</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1141,25 +1141,25 @@
         <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C24" t="n">
-        <v>21.87</v>
+        <v>22.78</v>
       </c>
       <c r="D24" t="n">
-        <v>52.33</v>
+        <v>52.43</v>
       </c>
       <c r="E24" t="n">
-        <v>3.48</v>
+        <v>2.74</v>
       </c>
       <c r="F24" t="n">
-        <v>0.57</v>
+        <v>0.6</v>
       </c>
       <c r="G24" t="n">
-        <v>-3.48</v>
+        <v>-2.74</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="s">
         <v>11</v>
@@ -1170,7 +1170,7 @@
         <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C25" t="n">
         <v>22.04</v>
@@ -1199,7 +1199,7 @@
         <v>20</v>
       </c>
       <c r="B26" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C26" t="n">
         <v>34.81</v>
@@ -1228,25 +1228,25 @@
         <v>20</v>
       </c>
       <c r="B27" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C27" t="n">
-        <v>33.35</v>
+        <v>24.59</v>
       </c>
       <c r="D27" t="n">
-        <v>79.56</v>
+        <v>63.37</v>
       </c>
       <c r="E27" t="n">
-        <v>1.38</v>
+        <v>0.96</v>
       </c>
       <c r="F27" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="G27" t="n">
-        <v>-1.38</v>
+        <v>-0.96</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="s">
         <v>11</v>
@@ -1257,25 +1257,25 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C28" t="n">
-        <v>24.59</v>
+        <v>38.87</v>
       </c>
       <c r="D28" t="n">
-        <v>63.37</v>
+        <v>98.87</v>
       </c>
       <c r="E28" t="n">
-        <v>0.96</v>
+        <v>1.36</v>
       </c>
       <c r="F28" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.96</v>
+        <v>-1.36</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" t="s">
         <v>11</v>
@@ -1286,7 +1286,7 @@
         <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C29" t="n">
         <v>36.23</v>
@@ -1318,19 +1318,19 @@
         <v>12</v>
       </c>
       <c r="C30" t="n">
-        <v>38.87</v>
+        <v>40.97</v>
       </c>
       <c r="D30" t="n">
-        <v>98.87</v>
+        <v>101.74</v>
       </c>
       <c r="E30" t="n">
-        <v>1.36</v>
+        <v>1.64</v>
       </c>
       <c r="F30" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="G30" t="n">
-        <v>-1.36</v>
+        <v>-1.64</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -1344,22 +1344,22 @@
         <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C31" t="n">
-        <v>40.2</v>
+        <v>32.81</v>
       </c>
       <c r="D31" t="n">
-        <v>96.77</v>
+        <v>78.78</v>
       </c>
       <c r="E31" t="n">
-        <v>1.83</v>
+        <v>1.34</v>
       </c>
       <c r="F31" t="n">
-        <v>0.49</v>
+        <v>0.66</v>
       </c>
       <c r="G31" t="n">
-        <v>-1.83</v>
+        <v>-1.34</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1373,22 +1373,22 @@
         <v>21</v>
       </c>
       <c r="B32" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C32" t="n">
-        <v>28.51</v>
+        <v>28.69</v>
       </c>
       <c r="D32" t="n">
-        <v>11.12</v>
+        <v>11.18</v>
       </c>
       <c r="E32" t="n">
-        <v>7.75</v>
+        <v>7.61</v>
       </c>
       <c r="F32" t="n">
-        <v>0.29</v>
+        <v>0.25</v>
       </c>
       <c r="G32" t="n">
-        <v>-7.75</v>
+        <v>-7.61</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1402,22 +1402,22 @@
         <v>21</v>
       </c>
       <c r="B33" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C33" t="n">
-        <v>30.34</v>
+        <v>31.22</v>
       </c>
       <c r="D33" t="n">
-        <v>11.83</v>
+        <v>12.67</v>
       </c>
       <c r="E33" t="n">
-        <v>2.47</v>
+        <v>7.11</v>
       </c>
       <c r="F33" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>-2.47</v>
+        <v>-7.11</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1431,25 +1431,25 @@
         <v>21</v>
       </c>
       <c r="B34" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C34" t="n">
-        <v>29.55</v>
+        <v>34.72</v>
       </c>
       <c r="D34" t="n">
-        <v>12.9</v>
+        <v>14.56</v>
       </c>
       <c r="E34" t="n">
-        <v>12.95</v>
+        <v>1.24</v>
       </c>
       <c r="F34" t="n">
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="G34" t="n">
-        <v>-12.95</v>
+        <v>-1.24</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" t="s">
         <v>11</v>
@@ -1460,25 +1460,19 @@
         <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C35" t="n">
-        <v>34.72</v>
+        <v>29.9</v>
       </c>
       <c r="D35" t="n">
-        <v>14.56</v>
-      </c>
-      <c r="E35" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G35" t="n">
-        <v>-1.24</v>
-      </c>
+        <v>12.07</v>
+      </c>
+      <c r="E35"/>
+      <c r="F35"/>
+      <c r="G35"/>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35" t="s">
         <v>11</v>
@@ -1492,14 +1486,20 @@
         <v>14</v>
       </c>
       <c r="C36" t="n">
-        <v>29.9</v>
+        <v>28.45</v>
       </c>
       <c r="D36" t="n">
-        <v>12.07</v>
-      </c>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
+        <v>11.04</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-3.51</v>
+      </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
@@ -1512,22 +1512,22 @@
         <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C37" t="n">
-        <v>28.45</v>
+        <v>30.34</v>
       </c>
       <c r="D37" t="n">
-        <v>11.04</v>
+        <v>11.83</v>
       </c>
       <c r="E37" t="n">
-        <v>3.51</v>
+        <v>2.47</v>
       </c>
       <c r="F37" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="G37" t="n">
-        <v>-3.51</v>
+        <v>-2.47</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -1544,22 +1544,22 @@
         <v>10</v>
       </c>
       <c r="C38" t="n">
-        <v>14.81</v>
+        <v>13.25</v>
       </c>
       <c r="D38" t="n">
-        <v>1990.08</v>
+        <v>1528.12</v>
       </c>
       <c r="E38" t="n">
-        <v>0.62</v>
+        <v>0.46</v>
       </c>
       <c r="F38" t="n">
         <v>0.96</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.62</v>
+        <v>-0.46</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="s">
         <v>23</v>
@@ -1570,25 +1570,25 @@
         <v>22</v>
       </c>
       <c r="B39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C39" t="n">
-        <v>13.25</v>
+        <v>14.81</v>
       </c>
       <c r="D39" t="n">
-        <v>1528.12</v>
+        <v>1990.08</v>
       </c>
       <c r="E39" t="n">
-        <v>0.46</v>
+        <v>0.62</v>
       </c>
       <c r="F39" t="n">
         <v>0.96</v>
       </c>
       <c r="G39" t="n">
-        <v>-0.46</v>
+        <v>-0.62</v>
       </c>
       <c r="H39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39" t="s">
         <v>23</v>
@@ -1602,19 +1602,19 @@
         <v>16</v>
       </c>
       <c r="C40" t="n">
-        <v>40.97</v>
+        <v>23.42</v>
       </c>
       <c r="D40" t="n">
-        <v>5545.28</v>
+        <v>3241.35</v>
       </c>
       <c r="E40" t="n">
-        <v>2.72</v>
+        <v>0.97</v>
       </c>
       <c r="F40" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="G40" t="n">
-        <v>-2.72</v>
+        <v>-0.97</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1628,7 +1628,7 @@
         <v>22</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C41" t="n">
         <v>79.5</v>
@@ -1657,22 +1657,22 @@
         <v>22</v>
       </c>
       <c r="B42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C42" t="n">
-        <v>21.83</v>
+        <v>40.97</v>
       </c>
       <c r="D42" t="n">
-        <v>3252.11</v>
+        <v>5545.28</v>
       </c>
       <c r="E42" t="n">
-        <v>1.11</v>
+        <v>2.72</v>
       </c>
       <c r="F42" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="G42" t="n">
-        <v>-1.11</v>
+        <v>-2.72</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1686,22 +1686,22 @@
         <v>22</v>
       </c>
       <c r="B43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C43" t="n">
-        <v>46.67</v>
+        <v>51.63</v>
       </c>
       <c r="D43" t="n">
-        <v>5151.77</v>
+        <v>5848.87</v>
       </c>
       <c r="E43" t="n">
-        <v>0.93</v>
+        <v>1.07</v>
       </c>
       <c r="F43" t="n">
-        <v>0.65</v>
+        <v>0.57</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.93</v>
+        <v>-1.07</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -1715,22 +1715,22 @@
         <v>24</v>
       </c>
       <c r="B44" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C44" t="n">
-        <v>31.44</v>
+        <v>27.92</v>
       </c>
       <c r="D44" t="n">
-        <v>73.25</v>
+        <v>69.61</v>
       </c>
       <c r="E44" t="n">
-        <v>1.68</v>
+        <v>1.71</v>
       </c>
       <c r="F44" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="G44" t="n">
-        <v>-1.68</v>
+        <v>-1.71</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -1744,22 +1744,22 @@
         <v>24</v>
       </c>
       <c r="B45" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C45" t="n">
-        <v>34.28</v>
+        <v>30.7</v>
       </c>
       <c r="D45" t="n">
-        <v>74.45</v>
+        <v>89.63</v>
       </c>
       <c r="E45" t="n">
-        <v>1.81</v>
+        <v>3.5</v>
       </c>
       <c r="F45" t="n">
-        <v>0.94</v>
+        <v>0.78</v>
       </c>
       <c r="G45" t="n">
-        <v>-1.81</v>
+        <v>-3.5</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -1773,22 +1773,22 @@
         <v>24</v>
       </c>
       <c r="B46" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C46" t="n">
-        <v>24.75</v>
+        <v>31.44</v>
       </c>
       <c r="D46" t="n">
-        <v>55.03</v>
+        <v>73.25</v>
       </c>
       <c r="E46" t="n">
-        <v>1.05</v>
+        <v>1.68</v>
       </c>
       <c r="F46" t="n">
-        <v>0.88</v>
+        <v>0.91</v>
       </c>
       <c r="G46" t="n">
-        <v>-1.05</v>
+        <v>-1.68</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -1805,19 +1805,19 @@
         <v>13</v>
       </c>
       <c r="C47" t="n">
-        <v>30.9</v>
+        <v>24.75</v>
       </c>
       <c r="D47" t="n">
-        <v>90.2</v>
+        <v>55.03</v>
       </c>
       <c r="E47" t="n">
-        <v>3.61</v>
+        <v>1.05</v>
       </c>
       <c r="F47" t="n">
-        <v>0.77</v>
+        <v>0.88</v>
       </c>
       <c r="G47" t="n">
-        <v>-3.61</v>
+        <v>-1.05</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -1831,7 +1831,7 @@
         <v>24</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C48" t="n">
         <v>22.95</v>
@@ -1860,22 +1860,22 @@
         <v>24</v>
       </c>
       <c r="B49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C49" t="n">
-        <v>27.8</v>
+        <v>34.28</v>
       </c>
       <c r="D49" t="n">
-        <v>67.83</v>
+        <v>74.45</v>
       </c>
       <c r="E49" t="n">
-        <v>1.6</v>
+        <v>1.81</v>
       </c>
       <c r="F49" t="n">
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="G49" t="n">
-        <v>-1.6</v>
+        <v>-1.81</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -1892,22 +1892,22 @@
         <v>14</v>
       </c>
       <c r="C50" t="n">
-        <v>12.11</v>
+        <v>20.33</v>
       </c>
       <c r="D50" t="n">
-        <v>100.91</v>
+        <v>185.53</v>
       </c>
       <c r="E50" t="n">
-        <v>0.6</v>
+        <v>1.04</v>
       </c>
       <c r="F50" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="G50" t="n">
-        <v>-0.6</v>
+        <v>-1.04</v>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I50" t="s">
         <v>23</v>
@@ -1918,22 +1918,22 @@
         <v>25</v>
       </c>
       <c r="B51" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C51" t="n">
-        <v>20.33</v>
+        <v>16.94</v>
       </c>
       <c r="D51" t="n">
-        <v>185.53</v>
+        <v>173.28</v>
       </c>
       <c r="E51" t="n">
-        <v>1.04</v>
+        <v>1.2</v>
       </c>
       <c r="F51" t="n">
-        <v>0.91</v>
+        <v>0.71</v>
       </c>
       <c r="G51" t="n">
-        <v>-1.04</v>
+        <v>-1.2</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -1947,25 +1947,25 @@
         <v>25</v>
       </c>
       <c r="B52" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C52" t="n">
-        <v>15.39</v>
+        <v>12.11</v>
       </c>
       <c r="D52" t="n">
-        <v>140.05</v>
+        <v>100.91</v>
       </c>
       <c r="E52" t="n">
-        <v>0.86</v>
+        <v>0.6</v>
       </c>
       <c r="F52" t="n">
-        <v>0.89</v>
+        <v>0.93</v>
       </c>
       <c r="G52" t="n">
-        <v>-0.86</v>
+        <v>-0.6</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="s">
         <v>23</v>
@@ -1976,22 +1976,22 @@
         <v>25</v>
       </c>
       <c r="B53" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C53" t="n">
-        <v>15.18</v>
+        <v>12.33</v>
       </c>
       <c r="D53" t="n">
-        <v>132.61</v>
+        <v>112.01</v>
       </c>
       <c r="E53" t="n">
-        <v>0.76</v>
+        <v>0.62</v>
       </c>
       <c r="F53" t="n">
         <v>0.92</v>
       </c>
       <c r="G53" t="n">
-        <v>-0.76</v>
+        <v>-0.62</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -2005,22 +2005,22 @@
         <v>25</v>
       </c>
       <c r="B54" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C54" t="n">
-        <v>12.33</v>
+        <v>15.18</v>
       </c>
       <c r="D54" t="n">
-        <v>112.01</v>
+        <v>132.61</v>
       </c>
       <c r="E54" t="n">
-        <v>0.62</v>
+        <v>0.76</v>
       </c>
       <c r="F54" t="n">
         <v>0.92</v>
       </c>
       <c r="G54" t="n">
-        <v>-0.62</v>
+        <v>-0.76</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -2034,22 +2034,22 @@
         <v>25</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C55" t="n">
-        <v>17.41</v>
+        <v>15.27</v>
       </c>
       <c r="D55" t="n">
-        <v>175.38</v>
+        <v>138.16</v>
       </c>
       <c r="E55" t="n">
-        <v>1.2</v>
+        <v>0.84</v>
       </c>
       <c r="F55" t="n">
-        <v>0.72</v>
+        <v>0.9</v>
       </c>
       <c r="G55" t="n">
-        <v>-1.2</v>
+        <v>-0.84</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -2066,22 +2066,22 @@
         <v>15</v>
       </c>
       <c r="C56" t="n">
-        <v>24.92</v>
+        <v>25.68</v>
       </c>
       <c r="D56" t="n">
-        <v>80.61</v>
+        <v>71.81</v>
       </c>
       <c r="E56" t="n">
-        <v>1.24</v>
+        <v>1.12</v>
       </c>
       <c r="F56" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="G56" t="n">
-        <v>-1.24</v>
+        <v>-1.12</v>
       </c>
       <c r="H56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I56" t="s">
         <v>23</v>
@@ -2092,7 +2092,7 @@
         <v>26</v>
       </c>
       <c r="B57" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C57" t="n">
         <v>26.57</v>
@@ -2121,22 +2121,22 @@
         <v>26</v>
       </c>
       <c r="B58" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C58" t="n">
-        <v>24.64</v>
+        <v>27.42</v>
       </c>
       <c r="D58" t="n">
-        <v>72.51</v>
+        <v>88.5</v>
       </c>
       <c r="E58" t="n">
-        <v>1.15</v>
+        <v>1.22</v>
       </c>
       <c r="F58" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="G58" t="n">
-        <v>-1.15</v>
+        <v>-1.22</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -2150,22 +2150,22 @@
         <v>26</v>
       </c>
       <c r="B59" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C59" t="n">
-        <v>27.42</v>
+        <v>24.64</v>
       </c>
       <c r="D59" t="n">
-        <v>83.15</v>
+        <v>72.51</v>
       </c>
       <c r="E59" t="n">
-        <v>1.42</v>
+        <v>1.15</v>
       </c>
       <c r="F59" t="n">
-        <v>0.73</v>
+        <v>0.62</v>
       </c>
       <c r="G59" t="n">
-        <v>-1.42</v>
+        <v>-1.15</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -2179,22 +2179,22 @@
         <v>26</v>
       </c>
       <c r="B60" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C60" t="n">
-        <v>27.42</v>
+        <v>26.77</v>
       </c>
       <c r="D60" t="n">
-        <v>88.5</v>
+        <v>82.1</v>
       </c>
       <c r="E60" t="n">
-        <v>1.22</v>
+        <v>1.42</v>
       </c>
       <c r="F60" t="n">
-        <v>0.59</v>
+        <v>0.68</v>
       </c>
       <c r="G60" t="n">
-        <v>-1.22</v>
+        <v>-1.42</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -2208,25 +2208,25 @@
         <v>26</v>
       </c>
       <c r="B61" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C61" t="n">
-        <v>25.68</v>
+        <v>25.07</v>
       </c>
       <c r="D61" t="n">
-        <v>71.81</v>
+        <v>80.24</v>
       </c>
       <c r="E61" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="F61" t="n">
         <v>0.63</v>
       </c>
       <c r="G61" t="n">
-        <v>-1.12</v>
+        <v>-1.22</v>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I61" t="s">
         <v>23</v>
@@ -2237,22 +2237,22 @@
         <v>27</v>
       </c>
       <c r="B62" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C62" t="n">
-        <v>10.8</v>
+        <v>20.46</v>
       </c>
       <c r="D62" t="n">
-        <v>29.7</v>
+        <v>45.6</v>
       </c>
       <c r="E62" t="n">
-        <v>1.9</v>
+        <v>1.49</v>
       </c>
       <c r="F62" t="n">
-        <v>0.75</v>
+        <v>0.88</v>
       </c>
       <c r="G62" t="n">
-        <v>-1.9</v>
+        <v>-1.49</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -2266,25 +2266,25 @@
         <v>27</v>
       </c>
       <c r="B63" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C63" t="n">
-        <v>19.8</v>
+        <v>9.97</v>
       </c>
       <c r="D63" t="n">
-        <v>45.1</v>
+        <v>26.23</v>
       </c>
       <c r="E63" t="n">
-        <v>1.34</v>
+        <v>1.48</v>
       </c>
       <c r="F63" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="G63" t="n">
-        <v>-1.34</v>
+        <v>-1.48</v>
       </c>
       <c r="H63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I63" t="s">
         <v>23</v>
@@ -2295,22 +2295,22 @@
         <v>27</v>
       </c>
       <c r="B64" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C64" t="n">
-        <v>16.98</v>
+        <v>21.03</v>
       </c>
       <c r="D64" t="n">
-        <v>39.92</v>
+        <v>46.49</v>
       </c>
       <c r="E64" t="n">
-        <v>1.42</v>
+        <v>1.4</v>
       </c>
       <c r="F64" t="n">
         <v>0.9</v>
       </c>
       <c r="G64" t="n">
-        <v>-1.42</v>
+        <v>-1.4</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2324,22 +2324,22 @@
         <v>27</v>
       </c>
       <c r="B65" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C65" t="n">
-        <v>21.03</v>
+        <v>23.51</v>
       </c>
       <c r="D65" t="n">
-        <v>46.49</v>
+        <v>52.04</v>
       </c>
       <c r="E65" t="n">
-        <v>1.4</v>
+        <v>1.64</v>
       </c>
       <c r="F65" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="G65" t="n">
-        <v>-1.4</v>
+        <v>-1.64</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -2356,22 +2356,22 @@
         <v>14</v>
       </c>
       <c r="C66" t="n">
-        <v>20.46</v>
+        <v>19.8</v>
       </c>
       <c r="D66" t="n">
-        <v>45.6</v>
+        <v>45.1</v>
       </c>
       <c r="E66" t="n">
-        <v>1.49</v>
+        <v>1.34</v>
       </c>
       <c r="F66" t="n">
-        <v>0.88</v>
+        <v>0.84</v>
       </c>
       <c r="G66" t="n">
-        <v>-1.49</v>
+        <v>-1.34</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66" t="s">
         <v>23</v>
@@ -2382,22 +2382,22 @@
         <v>27</v>
       </c>
       <c r="B67" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C67" t="n">
-        <v>23.51</v>
+        <v>15.79</v>
       </c>
       <c r="D67" t="n">
-        <v>52.04</v>
+        <v>37.89</v>
       </c>
       <c r="E67" t="n">
-        <v>1.64</v>
+        <v>1.37</v>
       </c>
       <c r="F67" t="n">
-        <v>0.82</v>
+        <v>0.91</v>
       </c>
       <c r="G67" t="n">
-        <v>-1.64</v>
+        <v>-1.37</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2411,22 +2411,22 @@
         <v>28</v>
       </c>
       <c r="B68" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C68" t="n">
-        <v>26.4</v>
+        <v>16.06</v>
       </c>
       <c r="D68" t="n">
-        <v>12.5</v>
+        <v>11.51</v>
       </c>
       <c r="E68" t="n">
-        <v>1.46</v>
+        <v>1.01</v>
       </c>
       <c r="F68" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="G68" t="n">
-        <v>-1.46</v>
+        <v>-1.01</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -2440,25 +2440,25 @@
         <v>28</v>
       </c>
       <c r="B69" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C69" t="n">
-        <v>17.11</v>
+        <v>29.15</v>
       </c>
       <c r="D69" t="n">
-        <v>10.16</v>
+        <v>13.39</v>
       </c>
       <c r="E69" t="n">
-        <v>0.9</v>
+        <v>1.81</v>
       </c>
       <c r="F69" t="n">
-        <v>0.8</v>
+        <v>0.73</v>
       </c>
       <c r="G69" t="n">
-        <v>-0.9</v>
+        <v>-1.81</v>
       </c>
       <c r="H69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I69" t="s">
         <v>23</v>
@@ -2469,25 +2469,25 @@
         <v>28</v>
       </c>
       <c r="B70" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C70" t="n">
-        <v>16.6</v>
+        <v>17.11</v>
       </c>
       <c r="D70" t="n">
-        <v>11.49</v>
+        <v>10.16</v>
       </c>
       <c r="E70" t="n">
-        <v>1.02</v>
+        <v>0.9</v>
       </c>
       <c r="F70" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="G70" t="n">
-        <v>-1.02</v>
+        <v>-0.9</v>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I70" t="s">
         <v>23</v>
@@ -2498,22 +2498,22 @@
         <v>28</v>
       </c>
       <c r="B71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C71" t="n">
-        <v>16.06</v>
+        <v>15</v>
       </c>
       <c r="D71" t="n">
-        <v>11.51</v>
+        <v>11.24</v>
       </c>
       <c r="E71" t="n">
-        <v>1.01</v>
+        <v>0.95</v>
       </c>
       <c r="F71" t="n">
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
       <c r="G71" t="n">
-        <v>-1.01</v>
+        <v>-0.95</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -2527,22 +2527,22 @@
         <v>28</v>
       </c>
       <c r="B72" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C72" t="n">
-        <v>15</v>
+        <v>15.58</v>
       </c>
       <c r="D72" t="n">
-        <v>11.24</v>
+        <v>11.31</v>
       </c>
       <c r="E72" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="G72" t="n">
-        <v>-0.95</v>
+        <v>-1</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
@@ -2559,19 +2559,19 @@
         <v>15</v>
       </c>
       <c r="C73" t="n">
-        <v>14.76</v>
+        <v>16.6</v>
       </c>
       <c r="D73" t="n">
-        <v>11.1</v>
+        <v>11.49</v>
       </c>
       <c r="E73" t="n">
-        <v>0.94</v>
+        <v>1.02</v>
       </c>
       <c r="F73" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="G73" t="n">
-        <v>-0.94</v>
+        <v>-1.02</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -2585,22 +2585,22 @@
         <v>29</v>
       </c>
       <c r="B74" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C74" t="n">
-        <v>42.31</v>
+        <v>30.54</v>
       </c>
       <c r="D74" t="n">
-        <v>3173.73</v>
+        <v>2016.4</v>
       </c>
       <c r="E74" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="F74" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="G74" t="n">
-        <v>-0.7</v>
+        <v>-0.85</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
@@ -2614,25 +2614,25 @@
         <v>29</v>
       </c>
       <c r="B75" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C75" t="n">
-        <v>27.57</v>
+        <v>32.83</v>
       </c>
       <c r="D75" t="n">
-        <v>1575.93</v>
+        <v>3120.22</v>
       </c>
       <c r="E75" t="n">
-        <v>0.44</v>
+        <v>1.56</v>
       </c>
       <c r="F75" t="n">
-        <v>0.96</v>
+        <v>0.75</v>
       </c>
       <c r="G75" t="n">
-        <v>-0.44</v>
+        <v>-1.56</v>
       </c>
       <c r="H75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I75" t="s">
         <v>30</v>
@@ -2646,19 +2646,19 @@
         <v>14</v>
       </c>
       <c r="C76" t="n">
-        <v>32.83</v>
+        <v>42.31</v>
       </c>
       <c r="D76" t="n">
-        <v>3120.22</v>
+        <v>3173.73</v>
       </c>
       <c r="E76" t="n">
-        <v>1.56</v>
+        <v>0.7</v>
       </c>
       <c r="F76" t="n">
-        <v>0.75</v>
+        <v>0.89</v>
       </c>
       <c r="G76" t="n">
-        <v>-1.56</v>
+        <v>-0.7</v>
       </c>
       <c r="H76" t="n">
         <v>0</v>
@@ -2675,19 +2675,19 @@
         <v>12</v>
       </c>
       <c r="C77" t="n">
-        <v>30.54</v>
+        <v>33.68</v>
       </c>
       <c r="D77" t="n">
-        <v>2016.4</v>
+        <v>3047.22</v>
       </c>
       <c r="E77" t="n">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="F77" t="n">
-        <v>0.84</v>
+        <v>0.78</v>
       </c>
       <c r="G77" t="n">
-        <v>-0.85</v>
+        <v>-0.63</v>
       </c>
       <c r="H77" t="n">
         <v>0</v>
@@ -2701,25 +2701,25 @@
         <v>29</v>
       </c>
       <c r="B78" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C78" t="n">
-        <v>33.63</v>
+        <v>31.16</v>
       </c>
       <c r="D78" t="n">
-        <v>2109.09</v>
+        <v>1895.72</v>
       </c>
       <c r="E78" t="n">
-        <v>0.92</v>
+        <v>0.61</v>
       </c>
       <c r="F78" t="n">
-        <v>0.79</v>
+        <v>0.83</v>
       </c>
       <c r="G78" t="n">
-        <v>-0.92</v>
+        <v>-0.61</v>
       </c>
       <c r="H78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I78" t="s">
         <v>30</v>
@@ -2730,22 +2730,22 @@
         <v>29</v>
       </c>
       <c r="B79" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C79" t="n">
-        <v>30.01</v>
+        <v>33.63</v>
       </c>
       <c r="D79" t="n">
-        <v>1756.65</v>
+        <v>2109.09</v>
       </c>
       <c r="E79" t="n">
-        <v>0.67</v>
+        <v>0.92</v>
       </c>
       <c r="F79" t="n">
-        <v>0.85</v>
+        <v>0.79</v>
       </c>
       <c r="G79" t="n">
-        <v>-0.67</v>
+        <v>-0.92</v>
       </c>
       <c r="H79" t="n">
         <v>0</v>
@@ -2759,22 +2759,22 @@
         <v>31</v>
       </c>
       <c r="B80" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C80" t="n">
-        <v>12.16</v>
+        <v>27.34</v>
       </c>
       <c r="D80" t="n">
-        <v>25.68</v>
+        <v>51.86</v>
       </c>
       <c r="E80" t="n">
-        <v>1.52</v>
+        <v>8.33</v>
       </c>
       <c r="F80" t="n">
-        <v>0.48</v>
+        <v>0.01</v>
       </c>
       <c r="G80" t="n">
-        <v>-1.52</v>
+        <v>-8.33</v>
       </c>
       <c r="H80" t="n">
         <v>0</v>
@@ -2791,22 +2791,22 @@
         <v>13</v>
       </c>
       <c r="C81" t="n">
-        <v>28.45</v>
+        <v>10.73</v>
       </c>
       <c r="D81" t="n">
-        <v>51.29</v>
+        <v>21.91</v>
       </c>
       <c r="E81" t="n">
-        <v>9.97</v>
+        <v>1.36</v>
       </c>
       <c r="F81" t="n">
-        <v>0.4</v>
+        <v>0.64</v>
       </c>
       <c r="G81" t="n">
-        <v>-9.97</v>
+        <v>-1.36</v>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I81" t="s">
         <v>30</v>
@@ -2820,19 +2820,19 @@
         <v>14</v>
       </c>
       <c r="C82" t="n">
-        <v>26.21</v>
+        <v>12.16</v>
       </c>
       <c r="D82" t="n">
-        <v>47.93</v>
+        <v>25.68</v>
       </c>
       <c r="E82" t="n">
-        <v>2.69</v>
+        <v>1.52</v>
       </c>
       <c r="F82" t="n">
-        <v>0.82</v>
+        <v>0.48</v>
       </c>
       <c r="G82" t="n">
-        <v>-2.69</v>
+        <v>-1.52</v>
       </c>
       <c r="H82" t="n">
         <v>0</v>
@@ -2846,7 +2846,7 @@
         <v>31</v>
       </c>
       <c r="B83" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C83" t="n">
         <v>29.78</v>
@@ -2878,22 +2878,22 @@
         <v>10</v>
       </c>
       <c r="C84" t="n">
-        <v>10.73</v>
+        <v>26.21</v>
       </c>
       <c r="D84" t="n">
-        <v>21.91</v>
+        <v>47.93</v>
       </c>
       <c r="E84" t="n">
-        <v>1.36</v>
+        <v>2.69</v>
       </c>
       <c r="F84" t="n">
-        <v>0.64</v>
+        <v>0.82</v>
       </c>
       <c r="G84" t="n">
-        <v>-1.36</v>
+        <v>-2.69</v>
       </c>
       <c r="H84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I84" t="s">
         <v>30</v>
@@ -2904,22 +2904,22 @@
         <v>31</v>
       </c>
       <c r="B85" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C85" t="n">
-        <v>18.56</v>
+        <v>19.15</v>
       </c>
       <c r="D85" t="n">
-        <v>33.26</v>
+        <v>34.25</v>
       </c>
       <c r="E85" t="n">
-        <v>2.71</v>
+        <v>3.06</v>
       </c>
       <c r="F85" t="n">
-        <v>0.67</v>
+        <v>0.6</v>
       </c>
       <c r="G85" t="n">
-        <v>-2.71</v>
+        <v>-3.06</v>
       </c>
       <c r="H85" t="n">
         <v>0</v>
@@ -2933,25 +2933,25 @@
         <v>32</v>
       </c>
       <c r="B86" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C86" t="n">
-        <v>35.17</v>
+        <v>20.57</v>
       </c>
       <c r="D86" t="n">
-        <v>28.81</v>
+        <v>19.83</v>
       </c>
       <c r="E86" t="n">
-        <v>3.27</v>
+        <v>1.78</v>
       </c>
       <c r="F86" t="n">
-        <v>0.6</v>
+        <v>0.49</v>
       </c>
       <c r="G86" t="n">
-        <v>-3.27</v>
+        <v>-1.78</v>
       </c>
       <c r="H86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I86" t="s">
         <v>30</v>
@@ -2962,22 +2962,22 @@
         <v>32</v>
       </c>
       <c r="B87" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C87" t="n">
-        <v>29.87</v>
+        <v>26.26</v>
       </c>
       <c r="D87" t="n">
-        <v>36.24</v>
+        <v>22.54</v>
       </c>
       <c r="E87" t="n">
-        <v>3.25</v>
+        <v>2.3</v>
       </c>
       <c r="F87" t="n">
-        <v>0.06</v>
+        <v>0.56</v>
       </c>
       <c r="G87" t="n">
-        <v>-3.25</v>
+        <v>-2.3</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
@@ -2991,25 +2991,25 @@
         <v>32</v>
       </c>
       <c r="B88" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C88" t="n">
-        <v>20.57</v>
+        <v>34.22</v>
       </c>
       <c r="D88" t="n">
-        <v>19.83</v>
+        <v>27.65</v>
       </c>
       <c r="E88" t="n">
-        <v>1.78</v>
+        <v>3.3</v>
       </c>
       <c r="F88" t="n">
-        <v>0.49</v>
+        <v>0.65</v>
       </c>
       <c r="G88" t="n">
-        <v>-1.78</v>
+        <v>-3.3</v>
       </c>
       <c r="H88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I88" t="s">
         <v>30</v>
@@ -3020,22 +3020,22 @@
         <v>32</v>
       </c>
       <c r="B89" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C89" t="n">
-        <v>26.26</v>
+        <v>35.17</v>
       </c>
       <c r="D89" t="n">
-        <v>22.54</v>
+        <v>28.81</v>
       </c>
       <c r="E89" t="n">
-        <v>2.3</v>
+        <v>3.27</v>
       </c>
       <c r="F89" t="n">
-        <v>0.56</v>
+        <v>0.6</v>
       </c>
       <c r="G89" t="n">
-        <v>-2.3</v>
+        <v>-3.27</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
@@ -3049,22 +3049,22 @@
         <v>32</v>
       </c>
       <c r="B90" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C90" t="n">
-        <v>30.9</v>
+        <v>25.93</v>
       </c>
       <c r="D90" t="n">
-        <v>26.24</v>
+        <v>25.63</v>
       </c>
       <c r="E90" t="n">
-        <v>3.54</v>
+        <v>3.89</v>
       </c>
       <c r="F90" t="n">
-        <v>0.4</v>
+        <v>0.06</v>
       </c>
       <c r="G90" t="n">
-        <v>-3.54</v>
+        <v>-3.89</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
@@ -3078,19 +3078,19 @@
         <v>32</v>
       </c>
       <c r="B91" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C91" t="n">
-        <v>34.22</v>
+        <v>29.31</v>
       </c>
       <c r="D91" t="n">
-        <v>27.65</v>
+        <v>24.97</v>
       </c>
       <c r="E91" t="n">
         <v>3.3</v>
       </c>
       <c r="F91" t="n">
-        <v>0.65</v>
+        <v>0.43</v>
       </c>
       <c r="G91" t="n">
         <v>-3.3</v>
@@ -3107,25 +3107,25 @@
         <v>33</v>
       </c>
       <c r="B92" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C92" t="n">
-        <v>15.95</v>
+        <v>27.26</v>
       </c>
       <c r="D92" t="n">
-        <v>18.2</v>
+        <v>29.44</v>
       </c>
       <c r="E92" t="n">
-        <v>1.23</v>
+        <v>1.82</v>
       </c>
       <c r="F92" t="n">
-        <v>0.39</v>
+        <v>0.69</v>
       </c>
       <c r="G92" t="n">
-        <v>-1.23</v>
+        <v>-1.82</v>
       </c>
       <c r="H92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I92" t="s">
         <v>30</v>
@@ -3136,22 +3136,22 @@
         <v>33</v>
       </c>
       <c r="B93" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C93" t="n">
-        <v>34.75</v>
+        <v>15.95</v>
       </c>
       <c r="D93" t="n">
-        <v>37.77</v>
+        <v>18.2</v>
       </c>
       <c r="E93" t="n">
-        <v>2.17</v>
+        <v>1.23</v>
       </c>
       <c r="F93" t="n">
-        <v>0.76</v>
+        <v>0.39</v>
       </c>
       <c r="G93" t="n">
-        <v>-2.17</v>
+        <v>-1.23</v>
       </c>
       <c r="H93" t="n">
         <v>0</v>
@@ -3165,22 +3165,22 @@
         <v>33</v>
       </c>
       <c r="B94" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C94" t="n">
-        <v>16.46</v>
+        <v>19.42</v>
       </c>
       <c r="D94" t="n">
-        <v>17.98</v>
+        <v>20.85</v>
       </c>
       <c r="E94" t="n">
-        <v>1.29</v>
+        <v>2.84</v>
       </c>
       <c r="F94" t="n">
-        <v>0.67</v>
+        <v>0.18</v>
       </c>
       <c r="G94" t="n">
-        <v>-1.29</v>
+        <v>-2.84</v>
       </c>
       <c r="H94" t="n">
         <v>0</v>
@@ -3194,25 +3194,25 @@
         <v>33</v>
       </c>
       <c r="B95" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C95" t="n">
-        <v>27.26</v>
+        <v>14.78</v>
       </c>
       <c r="D95" t="n">
-        <v>29.44</v>
+        <v>17.03</v>
       </c>
       <c r="E95" t="n">
-        <v>1.82</v>
+        <v>1.21</v>
       </c>
       <c r="F95" t="n">
-        <v>0.69</v>
+        <v>0.63</v>
       </c>
       <c r="G95" t="n">
-        <v>-1.82</v>
+        <v>-1.21</v>
       </c>
       <c r="H95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I95" t="s">
         <v>30</v>
@@ -3223,22 +3223,22 @@
         <v>33</v>
       </c>
       <c r="B96" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C96" t="n">
-        <v>19.35</v>
+        <v>34.75</v>
       </c>
       <c r="D96" t="n">
-        <v>20.86</v>
+        <v>37.77</v>
       </c>
       <c r="E96" t="n">
-        <v>2.74</v>
+        <v>2.17</v>
       </c>
       <c r="F96" t="n">
-        <v>0.18</v>
+        <v>0.76</v>
       </c>
       <c r="G96" t="n">
-        <v>-2.74</v>
+        <v>-2.17</v>
       </c>
       <c r="H96" t="n">
         <v>0</v>
@@ -3252,7 +3252,7 @@
         <v>33</v>
       </c>
       <c r="B97" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C97" t="n">
         <v>30.14</v>
@@ -3281,22 +3281,22 @@
         <v>34</v>
       </c>
       <c r="B98" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C98" t="n">
-        <v>11.01</v>
+        <v>11.58</v>
       </c>
       <c r="D98" t="n">
-        <v>5.01</v>
+        <v>5.47</v>
       </c>
       <c r="E98" t="n">
-        <v>3.8</v>
+        <v>0.91</v>
       </c>
       <c r="F98" t="n">
-        <v>0.17</v>
+        <v>0.24</v>
       </c>
       <c r="G98" t="n">
-        <v>-3.8</v>
+        <v>-0.91</v>
       </c>
       <c r="H98" t="n">
         <v>0</v>
@@ -3310,22 +3310,22 @@
         <v>34</v>
       </c>
       <c r="B99" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C99" t="n">
-        <v>8.89</v>
+        <v>10.22</v>
       </c>
       <c r="D99" t="n">
-        <v>3.5</v>
+        <v>4.78</v>
       </c>
       <c r="E99" t="n">
-        <v>0.69</v>
+        <v>1.73</v>
       </c>
       <c r="F99" t="n">
-        <v>0.63</v>
+        <v>0.19</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.69</v>
+        <v>-1.73</v>
       </c>
       <c r="H99" t="n">
         <v>0</v>
@@ -3339,25 +3339,25 @@
         <v>34</v>
       </c>
       <c r="B100" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C100" t="n">
-        <v>13.25</v>
+        <v>11.79</v>
       </c>
       <c r="D100" t="n">
-        <v>5.68</v>
+        <v>5.44</v>
       </c>
       <c r="E100" t="n">
-        <v>0.65</v>
+        <v>0.62</v>
       </c>
       <c r="F100" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.65</v>
+        <v>-0.62</v>
       </c>
       <c r="H100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I100" t="s">
         <v>30</v>
@@ -3368,22 +3368,22 @@
         <v>34</v>
       </c>
       <c r="B101" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C101" t="n">
-        <v>13.01</v>
+        <v>13.25</v>
       </c>
       <c r="D101" t="n">
-        <v>5.49</v>
+        <v>5.68</v>
       </c>
       <c r="E101" t="n">
-        <v>0.77</v>
+        <v>0.65</v>
       </c>
       <c r="F101" t="n">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
       <c r="G101" t="n">
-        <v>-0.77</v>
+        <v>-0.65</v>
       </c>
       <c r="H101" t="n">
         <v>0</v>
@@ -3397,25 +3397,25 @@
         <v>34</v>
       </c>
       <c r="B102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C102" t="n">
-        <v>11.79</v>
+        <v>13.01</v>
       </c>
       <c r="D102" t="n">
-        <v>5.44</v>
+        <v>5.49</v>
       </c>
       <c r="E102" t="n">
-        <v>0.62</v>
+        <v>0.77</v>
       </c>
       <c r="F102" t="n">
-        <v>0.72</v>
+        <v>0.52</v>
       </c>
       <c r="G102" t="n">
-        <v>-0.62</v>
+        <v>-0.77</v>
       </c>
       <c r="H102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I102" t="s">
         <v>30</v>
@@ -3429,19 +3429,19 @@
         <v>16</v>
       </c>
       <c r="C103" t="n">
-        <v>11.58</v>
+        <v>8.08</v>
       </c>
       <c r="D103" t="n">
-        <v>5.47</v>
+        <v>3.19</v>
       </c>
       <c r="E103" t="n">
-        <v>0.91</v>
+        <v>0.84</v>
       </c>
       <c r="F103" t="n">
-        <v>0.24</v>
+        <v>0.6</v>
       </c>
       <c r="G103" t="n">
-        <v>-0.91</v>
+        <v>-0.84</v>
       </c>
       <c r="H103" t="n">
         <v>0</v>
@@ -3455,22 +3455,22 @@
         <v>35</v>
       </c>
       <c r="B104" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C104" t="n">
-        <v>9.47</v>
+        <v>13.48</v>
       </c>
       <c r="D104" t="n">
-        <v>90.13</v>
+        <v>127.7</v>
       </c>
       <c r="E104" t="n">
-        <v>1.75</v>
+        <v>2.12</v>
       </c>
       <c r="F104" t="n">
         <v>0.54</v>
       </c>
       <c r="G104" t="n">
-        <v>-1.75</v>
+        <v>-2.12</v>
       </c>
       <c r="H104" t="n">
         <v>0</v>
@@ -3484,22 +3484,22 @@
         <v>35</v>
       </c>
       <c r="B105" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C105" t="n">
-        <v>13.48</v>
+        <v>6.09</v>
       </c>
       <c r="D105" t="n">
-        <v>127.7</v>
+        <v>60.99</v>
       </c>
       <c r="E105" t="n">
-        <v>2.12</v>
+        <v>4.98</v>
       </c>
       <c r="F105" t="n">
-        <v>0.54</v>
+        <v>0.59</v>
       </c>
       <c r="G105" t="n">
-        <v>-2.12</v>
+        <v>-4.98</v>
       </c>
       <c r="H105" t="n">
         <v>0</v>
@@ -3513,7 +3513,7 @@
         <v>35</v>
       </c>
       <c r="B106" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C106" t="n">
         <v>10.79</v>
@@ -3542,7 +3542,7 @@
         <v>35</v>
       </c>
       <c r="B107" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C107" t="n">
         <v>14.76</v>
@@ -3574,22 +3574,22 @@
         <v>13</v>
       </c>
       <c r="C108" t="n">
-        <v>7.47</v>
+        <v>8.82</v>
       </c>
       <c r="D108" t="n">
-        <v>68.59</v>
+        <v>88.54</v>
       </c>
       <c r="E108" t="n">
-        <v>6.06</v>
+        <v>1.16</v>
       </c>
       <c r="F108" t="n">
-        <v>0.37</v>
+        <v>0.44</v>
       </c>
       <c r="G108" t="n">
-        <v>-6.06</v>
+        <v>-1.16</v>
       </c>
       <c r="H108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I108" t="s">
         <v>36</v>
@@ -3600,25 +3600,25 @@
         <v>35</v>
       </c>
       <c r="B109" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C109" t="n">
-        <v>8.82</v>
+        <v>9.44</v>
       </c>
       <c r="D109" t="n">
-        <v>88.54</v>
+        <v>90.42</v>
       </c>
       <c r="E109" t="n">
-        <v>1.16</v>
+        <v>1.67</v>
       </c>
       <c r="F109" t="n">
-        <v>0.44</v>
+        <v>0.53</v>
       </c>
       <c r="G109" t="n">
-        <v>-1.16</v>
+        <v>-1.67</v>
       </c>
       <c r="H109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I109" t="s">
         <v>36</v>
@@ -3629,25 +3629,25 @@
         <v>37</v>
       </c>
       <c r="B110" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C110" t="n">
-        <v>4.57</v>
+        <v>38.29</v>
       </c>
       <c r="D110" t="n">
-        <v>43.36</v>
+        <v>508.07</v>
       </c>
       <c r="E110" t="n">
-        <v>0.43</v>
+        <v>1.08</v>
       </c>
       <c r="F110" t="n">
-        <v>0.78</v>
+        <v>0.42</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.43</v>
+        <v>-1.08</v>
       </c>
       <c r="H110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I110" t="s">
         <v>36</v>
@@ -3658,25 +3658,25 @@
         <v>37</v>
       </c>
       <c r="B111" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C111" t="n">
-        <v>12.87</v>
+        <v>4.57</v>
       </c>
       <c r="D111" t="n">
-        <v>110.82</v>
+        <v>43.36</v>
       </c>
       <c r="E111" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G111" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="H111" t="n">
         <v>1</v>
-      </c>
-      <c r="F111" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="G111" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H111" t="n">
-        <v>0</v>
       </c>
       <c r="I111" t="s">
         <v>36</v>
@@ -3687,22 +3687,22 @@
         <v>37</v>
       </c>
       <c r="B112" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C112" t="n">
-        <v>56.07</v>
+        <v>10.01</v>
       </c>
       <c r="D112" t="n">
-        <v>853.08</v>
+        <v>104.79</v>
       </c>
       <c r="E112" t="n">
-        <v>1.21</v>
+        <v>0.71</v>
       </c>
       <c r="F112" t="n">
-        <v>0.39</v>
+        <v>0.53</v>
       </c>
       <c r="G112" t="n">
-        <v>-1.21</v>
+        <v>-0.71</v>
       </c>
       <c r="H112" t="n">
         <v>0</v>
@@ -3716,22 +3716,22 @@
         <v>37</v>
       </c>
       <c r="B113" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C113" t="n">
-        <v>11.62</v>
+        <v>12.87</v>
       </c>
       <c r="D113" t="n">
-        <v>95.18</v>
+        <v>110.82</v>
       </c>
       <c r="E113" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F113" t="n">
-        <v>0.47</v>
+        <v>0.28</v>
       </c>
       <c r="G113" t="n">
-        <v>-0.95</v>
+        <v>-1</v>
       </c>
       <c r="H113" t="n">
         <v>0</v>
@@ -3745,22 +3745,22 @@
         <v>37</v>
       </c>
       <c r="B114" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C114" t="n">
-        <v>10.44</v>
+        <v>11.62</v>
       </c>
       <c r="D114" t="n">
-        <v>119.9</v>
+        <v>95.18</v>
       </c>
       <c r="E114" t="n">
-        <v>0.72</v>
+        <v>0.95</v>
       </c>
       <c r="F114" t="n">
-        <v>0.51</v>
+        <v>0.47</v>
       </c>
       <c r="G114" t="n">
-        <v>-0.72</v>
+        <v>-0.95</v>
       </c>
       <c r="H114" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
         <v>37</v>
       </c>
       <c r="B115" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C115" t="n">
         <v>13.28</v>
@@ -3803,22 +3803,22 @@
         <v>38</v>
       </c>
       <c r="B116" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C116" t="n">
-        <v>8.64</v>
+        <v>8.38</v>
       </c>
       <c r="D116" t="n">
-        <v>63.09</v>
+        <v>63.81</v>
       </c>
       <c r="E116" t="n">
-        <v>0.84</v>
+        <v>0.67</v>
       </c>
       <c r="F116" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="G116" t="n">
-        <v>-0.84</v>
+        <v>-0.67</v>
       </c>
       <c r="H116" t="n">
         <v>0</v>
@@ -3835,19 +3835,19 @@
         <v>14</v>
       </c>
       <c r="C117" t="n">
-        <v>7.74</v>
+        <v>8.64</v>
       </c>
       <c r="D117" t="n">
-        <v>58.69</v>
+        <v>63.09</v>
       </c>
       <c r="E117" t="n">
-        <v>0.72</v>
+        <v>0.84</v>
       </c>
       <c r="F117" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="G117" t="n">
-        <v>-0.72</v>
+        <v>-0.84</v>
       </c>
       <c r="H117" t="n">
         <v>0</v>
@@ -3861,22 +3861,22 @@
         <v>38</v>
       </c>
       <c r="B118" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C118" t="n">
-        <v>8.38</v>
+        <v>7.57</v>
       </c>
       <c r="D118" t="n">
-        <v>63.81</v>
+        <v>60.99</v>
       </c>
       <c r="E118" t="n">
-        <v>0.67</v>
+        <v>0.63</v>
       </c>
       <c r="F118" t="n">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="G118" t="n">
-        <v>-0.67</v>
+        <v>-0.63</v>
       </c>
       <c r="H118" t="n">
         <v>0</v>
@@ -3893,19 +3893,19 @@
         <v>10</v>
       </c>
       <c r="C119" t="n">
-        <v>7.57</v>
+        <v>7.74</v>
       </c>
       <c r="D119" t="n">
-        <v>60.99</v>
+        <v>58.69</v>
       </c>
       <c r="E119" t="n">
-        <v>0.63</v>
+        <v>0.72</v>
       </c>
       <c r="F119" t="n">
-        <v>0.81</v>
+        <v>0.85</v>
       </c>
       <c r="G119" t="n">
-        <v>-0.63</v>
+        <v>-0.72</v>
       </c>
       <c r="H119" t="n">
         <v>0</v>
@@ -3919,25 +3919,25 @@
         <v>38</v>
       </c>
       <c r="B120" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C120" t="n">
-        <v>6.81</v>
+        <v>8.15</v>
       </c>
       <c r="D120" t="n">
-        <v>56.71</v>
+        <v>61.36</v>
       </c>
       <c r="E120" t="n">
-        <v>0.56</v>
+        <v>0.53</v>
       </c>
       <c r="F120" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="G120" t="n">
-        <v>-0.56</v>
+        <v>-0.53</v>
       </c>
       <c r="H120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I120" t="s">
         <v>36</v>
@@ -3948,25 +3948,25 @@
         <v>38</v>
       </c>
       <c r="B121" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C121" t="n">
-        <v>8.29</v>
+        <v>7.18</v>
       </c>
       <c r="D121" t="n">
-        <v>65.58</v>
+        <v>57.42</v>
       </c>
       <c r="E121" t="n">
-        <v>0.48</v>
+        <v>0.62</v>
       </c>
       <c r="F121" t="n">
-        <v>0.63</v>
+        <v>0.84</v>
       </c>
       <c r="G121" t="n">
-        <v>-0.48</v>
+        <v>-0.62</v>
       </c>
       <c r="H121" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I121" t="s">
         <v>36</v>
@@ -3980,19 +3980,19 @@
         <v>15</v>
       </c>
       <c r="C122" t="n">
-        <v>8.84</v>
+        <v>8.66</v>
       </c>
       <c r="D122" t="n">
-        <v>38.28</v>
+        <v>37.72</v>
       </c>
       <c r="E122" t="n">
-        <v>1.17</v>
+        <v>0.9</v>
       </c>
       <c r="F122" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="G122" t="n">
-        <v>-1.17</v>
+        <v>-0.9</v>
       </c>
       <c r="H122" t="n">
         <v>0</v>
@@ -4006,7 +4006,7 @@
         <v>39</v>
       </c>
       <c r="B123" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C123" t="n">
         <v>12.49</v>
@@ -4035,25 +4035,25 @@
         <v>39</v>
       </c>
       <c r="B124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C124" t="n">
-        <v>9.25</v>
+        <v>9.32</v>
       </c>
       <c r="D124" t="n">
-        <v>39.98</v>
+        <v>42.19</v>
       </c>
       <c r="E124" t="n">
-        <v>1.08</v>
+        <v>0.89</v>
       </c>
       <c r="F124" t="n">
-        <v>0.68</v>
+        <v>0.55</v>
       </c>
       <c r="G124" t="n">
-        <v>-1.08</v>
+        <v>-0.89</v>
       </c>
       <c r="H124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I124" t="s">
         <v>36</v>
@@ -4067,19 +4067,19 @@
         <v>12</v>
       </c>
       <c r="C125" t="n">
-        <v>8.66</v>
+        <v>7.84</v>
       </c>
       <c r="D125" t="n">
-        <v>37.72</v>
+        <v>34.29</v>
       </c>
       <c r="E125" t="n">
-        <v>0.9</v>
+        <v>1.47</v>
       </c>
       <c r="F125" t="n">
-        <v>0.71</v>
+        <v>0.85</v>
       </c>
       <c r="G125" t="n">
-        <v>-0.9</v>
+        <v>-1.47</v>
       </c>
       <c r="H125" t="n">
         <v>0</v>
@@ -4093,22 +4093,22 @@
         <v>39</v>
       </c>
       <c r="B126" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C126" t="n">
-        <v>8.31</v>
+        <v>9.25</v>
       </c>
       <c r="D126" t="n">
-        <v>37.94</v>
+        <v>39.98</v>
       </c>
       <c r="E126" t="n">
-        <v>1.53</v>
+        <v>1.08</v>
       </c>
       <c r="F126" t="n">
-        <v>0.81</v>
+        <v>0.68</v>
       </c>
       <c r="G126" t="n">
-        <v>-1.53</v>
+        <v>-1.08</v>
       </c>
       <c r="H126" t="n">
         <v>0</v>
@@ -4122,25 +4122,25 @@
         <v>39</v>
       </c>
       <c r="B127" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C127" t="n">
-        <v>9.32</v>
+        <v>8</v>
       </c>
       <c r="D127" t="n">
-        <v>42.19</v>
+        <v>34.97</v>
       </c>
       <c r="E127" t="n">
-        <v>0.89</v>
+        <v>1.17</v>
       </c>
       <c r="F127" t="n">
-        <v>0.55</v>
+        <v>0.78</v>
       </c>
       <c r="G127" t="n">
-        <v>-0.89</v>
+        <v>-1.17</v>
       </c>
       <c r="H127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I127" t="s">
         <v>36</v>
@@ -4151,25 +4151,25 @@
         <v>40</v>
       </c>
       <c r="B128" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C128" t="n">
-        <v>12.77</v>
+        <v>6.88</v>
       </c>
       <c r="D128" t="n">
-        <v>24.9</v>
+        <v>16.38</v>
       </c>
       <c r="E128" t="n">
-        <v>1.39</v>
+        <v>4.73</v>
       </c>
       <c r="F128" t="n">
-        <v>0.01</v>
+        <v>0.13</v>
       </c>
       <c r="G128" t="n">
-        <v>-1.39</v>
+        <v>-4.73</v>
       </c>
       <c r="H128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I128" t="s">
         <v>36</v>
@@ -4180,22 +4180,22 @@
         <v>40</v>
       </c>
       <c r="B129" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C129" t="n">
-        <v>15.61</v>
+        <v>9.59</v>
       </c>
       <c r="D129" t="n">
-        <v>29.31</v>
+        <v>19.02</v>
       </c>
       <c r="E129" t="n">
-        <v>1.66</v>
+        <v>1.81</v>
       </c>
       <c r="F129" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="G129" t="n">
-        <v>-1.66</v>
+        <v>-1.81</v>
       </c>
       <c r="H129" t="n">
         <v>0</v>
@@ -4209,22 +4209,22 @@
         <v>40</v>
       </c>
       <c r="B130" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C130" t="n">
-        <v>8.05</v>
+        <v>15.61</v>
       </c>
       <c r="D130" t="n">
-        <v>16.82</v>
+        <v>29.31</v>
       </c>
       <c r="E130" t="n">
-        <v>1.82</v>
+        <v>1.66</v>
       </c>
       <c r="F130" t="n">
-        <v>0.07</v>
+        <v>0.02</v>
       </c>
       <c r="G130" t="n">
-        <v>-1.82</v>
+        <v>-1.66</v>
       </c>
       <c r="H130" t="n">
         <v>0</v>
@@ -4238,25 +4238,25 @@
         <v>40</v>
       </c>
       <c r="B131" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>9.97</v>
+        <v>12.77</v>
       </c>
       <c r="D131" t="n">
-        <v>19.56</v>
+        <v>24.9</v>
       </c>
       <c r="E131" t="n">
-        <v>1.77</v>
+        <v>1.39</v>
       </c>
       <c r="F131" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="G131" t="n">
-        <v>-1.77</v>
+        <v>-1.39</v>
       </c>
       <c r="H131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I131" t="s">
         <v>36</v>
@@ -4267,7 +4267,7 @@
         <v>40</v>
       </c>
       <c r="B132" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C132" t="n">
         <v>13.52</v>
@@ -4296,22 +4296,22 @@
         <v>40</v>
       </c>
       <c r="B133" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C133" t="n">
-        <v>6.93</v>
+        <v>8.05</v>
       </c>
       <c r="D133" t="n">
-        <v>16.43</v>
+        <v>16.82</v>
       </c>
       <c r="E133" t="n">
-        <v>4.86</v>
+        <v>1.82</v>
       </c>
       <c r="F133" t="n">
-        <v>0.11</v>
+        <v>0.07</v>
       </c>
       <c r="G133" t="n">
-        <v>-4.86</v>
+        <v>-1.82</v>
       </c>
       <c r="H133" t="n">
         <v>0</v>
@@ -4325,25 +4325,25 @@
         <v>41</v>
       </c>
       <c r="B134" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C134" t="n">
-        <v>7.62</v>
+        <v>10.21</v>
       </c>
       <c r="D134" t="n">
-        <v>9.93</v>
+        <v>13.77</v>
       </c>
       <c r="E134" t="n">
-        <v>0.98</v>
+        <v>2.78</v>
       </c>
       <c r="F134" t="n">
-        <v>0.07</v>
+        <v>0.01</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.98</v>
+        <v>-2.78</v>
       </c>
       <c r="H134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I134" t="s">
         <v>36</v>
@@ -4354,22 +4354,22 @@
         <v>41</v>
       </c>
       <c r="B135" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C135" t="n">
-        <v>16.2</v>
+        <v>11.73</v>
       </c>
       <c r="D135" t="n">
-        <v>20.69</v>
+        <v>15.01</v>
       </c>
       <c r="E135" t="n">
-        <v>1.85</v>
+        <v>2.46</v>
       </c>
       <c r="F135" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="G135" t="n">
-        <v>-1.85</v>
+        <v>-2.46</v>
       </c>
       <c r="H135" t="n">
         <v>0</v>
@@ -4383,7 +4383,7 @@
         <v>41</v>
       </c>
       <c r="B136" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C136" t="n">
         <v>15.89</v>
@@ -4412,25 +4412,25 @@
         <v>41</v>
       </c>
       <c r="B137" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C137" t="n">
-        <v>10.47</v>
+        <v>7.66</v>
       </c>
       <c r="D137" t="n">
-        <v>13.55</v>
+        <v>9.9</v>
       </c>
       <c r="E137" t="n">
-        <v>2.29</v>
+        <v>1.02</v>
       </c>
       <c r="F137" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G137" t="n">
-        <v>-2.29</v>
+        <v>-1.02</v>
       </c>
       <c r="H137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I137" t="s">
         <v>36</v>
@@ -4441,22 +4441,22 @@
         <v>41</v>
       </c>
       <c r="B138" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C138" t="n">
-        <v>16.54</v>
+        <v>16.2</v>
       </c>
       <c r="D138" t="n">
-        <v>20.79</v>
+        <v>20.69</v>
       </c>
       <c r="E138" t="n">
-        <v>2.53</v>
+        <v>1.85</v>
       </c>
       <c r="F138" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="G138" t="n">
-        <v>-2.53</v>
+        <v>-1.85</v>
       </c>
       <c r="H138" t="n">
         <v>0</v>
@@ -4470,22 +4470,22 @@
         <v>41</v>
       </c>
       <c r="B139" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C139" t="n">
-        <v>10.21</v>
+        <v>16.54</v>
       </c>
       <c r="D139" t="n">
-        <v>13.77</v>
+        <v>20.79</v>
       </c>
       <c r="E139" t="n">
-        <v>2.78</v>
+        <v>2.53</v>
       </c>
       <c r="F139" t="n">
-        <v>0.01</v>
+        <v>0.14</v>
       </c>
       <c r="G139" t="n">
-        <v>-2.78</v>
+        <v>-2.53</v>
       </c>
       <c r="H139" t="n">
         <v>0</v>
@@ -4499,22 +4499,22 @@
         <v>42</v>
       </c>
       <c r="B140" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C140" t="n">
-        <v>71.22</v>
+        <v>27.09</v>
       </c>
       <c r="D140" t="n">
-        <v>28.25</v>
+        <v>16.65</v>
       </c>
       <c r="E140" t="n">
-        <v>6.98</v>
+        <v>2.15</v>
       </c>
       <c r="F140" t="n">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="G140" t="n">
-        <v>-6.98</v>
+        <v>-2.15</v>
       </c>
       <c r="H140" t="n">
         <v>0</v>
@@ -4528,22 +4528,22 @@
         <v>42</v>
       </c>
       <c r="B141" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C141" t="n">
-        <v>30.24</v>
+        <v>66.51</v>
       </c>
       <c r="D141" t="n">
-        <v>18.68</v>
+        <v>27.62</v>
       </c>
       <c r="E141" t="n">
-        <v>3.17</v>
+        <v>3.88</v>
       </c>
       <c r="F141" t="n">
-        <v>0.51</v>
+        <v>0.01</v>
       </c>
       <c r="G141" t="n">
-        <v>-3.17</v>
+        <v>-3.88</v>
       </c>
       <c r="H141" t="n">
         <v>0</v>
@@ -4557,25 +4557,25 @@
         <v>42</v>
       </c>
       <c r="B142" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C142" t="n">
-        <v>26.44</v>
+        <v>26.52</v>
       </c>
       <c r="D142" t="n">
-        <v>14.18</v>
+        <v>14.53</v>
       </c>
       <c r="E142" t="n">
-        <v>2.03</v>
+        <v>2.09</v>
       </c>
       <c r="F142" t="n">
-        <v>0.68</v>
+        <v>0.73</v>
       </c>
       <c r="G142" t="n">
-        <v>-2.03</v>
+        <v>-2.09</v>
       </c>
       <c r="H142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I142" t="s">
         <v>36</v>
@@ -4586,25 +4586,25 @@
         <v>42</v>
       </c>
       <c r="B143" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C143" t="n">
-        <v>27.21</v>
+        <v>26.44</v>
       </c>
       <c r="D143" t="n">
-        <v>16.4</v>
+        <v>14.18</v>
       </c>
       <c r="E143" t="n">
-        <v>2.34</v>
+        <v>2.03</v>
       </c>
       <c r="F143" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="G143" t="n">
-        <v>-2.34</v>
+        <v>-2.03</v>
       </c>
       <c r="H143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I143" t="s">
         <v>36</v>
@@ -4615,22 +4615,22 @@
         <v>42</v>
       </c>
       <c r="B144" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C144" t="n">
-        <v>26.52</v>
+        <v>27.21</v>
       </c>
       <c r="D144" t="n">
-        <v>14.53</v>
+        <v>16.4</v>
       </c>
       <c r="E144" t="n">
-        <v>2.09</v>
+        <v>2.34</v>
       </c>
       <c r="F144" t="n">
-        <v>0.73</v>
+        <v>0.58</v>
       </c>
       <c r="G144" t="n">
-        <v>-2.09</v>
+        <v>-2.34</v>
       </c>
       <c r="H144" t="n">
         <v>0</v>
@@ -4647,19 +4647,19 @@
         <v>16</v>
       </c>
       <c r="C145" t="n">
-        <v>27.09</v>
+        <v>31.99</v>
       </c>
       <c r="D145" t="n">
-        <v>16.65</v>
+        <v>19.27</v>
       </c>
       <c r="E145" t="n">
-        <v>2.15</v>
+        <v>3.12</v>
       </c>
       <c r="F145" t="n">
-        <v>0.53</v>
+        <v>0.42</v>
       </c>
       <c r="G145" t="n">
-        <v>-2.15</v>
+        <v>-3.12</v>
       </c>
       <c r="H145" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
using MCMC method create figure 4 trend
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Best_model_outcome.xlsx
+++ b/Outcome/Appendix/Best_model_outcome.xlsx
@@ -482,7 +482,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>3.45</v>
+        <v>2.9</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -499,7 +499,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>7.48</v>
+        <v>7.44</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -516,7 +516,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.84</v>
+        <v>-1.3</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -533,7 +533,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>-13.43</v>
+        <v>-11.78</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -550,7 +550,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>-2.1</v>
+        <v>-2.79</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -567,7 +567,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>5.44</v>
+        <v>5.53</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -584,7 +584,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.07</v>
+        <v>-0.61</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -601,7 +601,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.97</v>
+        <v>1.19</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -618,7 +618,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>2.91</v>
+        <v>1.92</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -635,7 +635,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.87</v>
+        <v>0.63</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.19</v>
+        <v>-0.82</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -669,7 +669,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>-2.75</v>
+        <v>-2.31</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -686,7 +686,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>-4.12</v>
+        <v>-4.02</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -703,7 +703,7 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>2.97</v>
+        <v>3.07</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -720,7 +720,7 @@
         <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>3.72</v>
+        <v>3.99</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -737,7 +737,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>-3.98</v>
+        <v>-4.78</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -754,7 +754,7 @@
         <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.22</v>
+        <v>-0.01</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -771,7 +771,7 @@
         <v>12</v>
       </c>
       <c r="C19" t="n">
-        <v>1.63</v>
+        <v>1.75</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>8.64</v>
+        <v>9.16</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
@@ -805,7 +805,7 @@
         <v>8</v>
       </c>
       <c r="C21" t="n">
-        <v>-2.64</v>
+        <v>-2.57</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -822,7 +822,7 @@
         <v>9</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.61</v>
+        <v>-1.1</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -839,7 +839,7 @@
         <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>3.06</v>
+        <v>2.93</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>11</v>
       </c>
       <c r="C24" t="n">
-        <v>-11.78</v>
+        <v>-12.1</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -873,7 +873,7 @@
         <v>12</v>
       </c>
       <c r="C25" t="n">
-        <v>3.33</v>
+        <v>3.67</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -890,7 +890,7 @@
         <v>6</v>
       </c>
       <c r="C26" t="n">
-        <v>1.95</v>
+        <v>2.29</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -907,7 +907,7 @@
         <v>8</v>
       </c>
       <c r="C27" t="n">
-        <v>2.66</v>
+        <v>2.92</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -924,7 +924,7 @@
         <v>9</v>
       </c>
       <c r="C28" t="n">
-        <v>5.07</v>
+        <v>4.85</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
@@ -941,7 +941,7 @@
         <v>10</v>
       </c>
       <c r="C29" t="n">
-        <v>-10.52</v>
+        <v>-11.78</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -958,7 +958,7 @@
         <v>11</v>
       </c>
       <c r="C30" t="n">
-        <v>-0.43</v>
+        <v>0.07</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
         <v>12</v>
       </c>
       <c r="C31" t="n">
-        <v>1.28</v>
+        <v>1.64</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -992,7 +992,7 @@
         <v>6</v>
       </c>
       <c r="C32" t="n">
-        <v>8.07</v>
+        <v>8.35</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
@@ -1009,7 +1009,7 @@
         <v>8</v>
       </c>
       <c r="C33" t="n">
-        <v>1.31</v>
+        <v>1.47</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1026,7 +1026,7 @@
         <v>9</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.45</v>
+        <v>-0.07</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
         <v>10</v>
       </c>
       <c r="C35" t="n">
-        <v>-13.48</v>
+        <v>-14.08</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1060,7 +1060,7 @@
         <v>11</v>
       </c>
       <c r="C36" t="n">
-        <v>4.53</v>
+        <v>4.06</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>12</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01</v>
+        <v>0.27</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1094,7 +1094,7 @@
         <v>6</v>
       </c>
       <c r="C38" t="n">
-        <v>-5.97</v>
+        <v>-6.06</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -1111,7 +1111,7 @@
         <v>8</v>
       </c>
       <c r="C39" t="n">
-        <v>3.47</v>
+        <v>3.81</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1128,7 +1128,7 @@
         <v>9</v>
       </c>
       <c r="C40" t="n">
-        <v>3.36</v>
+        <v>4.03</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1145,7 +1145,7 @@
         <v>10</v>
       </c>
       <c r="C41" t="n">
-        <v>1.32</v>
+        <v>0.02</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1162,7 +1162,7 @@
         <v>11</v>
       </c>
       <c r="C42" t="n">
-        <v>-8.76</v>
+        <v>-8.79</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -1179,7 +1179,7 @@
         <v>12</v>
       </c>
       <c r="C43" t="n">
-        <v>6.59</v>
+        <v>6.98</v>
       </c>
       <c r="D43" t="n">
         <v>1</v>
@@ -1196,7 +1196,7 @@
         <v>6</v>
       </c>
       <c r="C44" t="n">
-        <v>-3.03</v>
+        <v>-4.09</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1213,7 +1213,7 @@
         <v>8</v>
       </c>
       <c r="C45" t="n">
-        <v>-1.05</v>
+        <v>-0.94</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1230,7 +1230,7 @@
         <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>8.19</v>
+        <v>9.07</v>
       </c>
       <c r="D46" t="n">
         <v>1</v>
@@ -1247,7 +1247,7 @@
         <v>10</v>
       </c>
       <c r="C47" t="n">
-        <v>-5.73</v>
+        <v>-5.9</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
@@ -1264,7 +1264,7 @@
         <v>11</v>
       </c>
       <c r="C48" t="n">
-        <v>-0.61</v>
+        <v>-0.18</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -1281,7 +1281,7 @@
         <v>12</v>
       </c>
       <c r="C49" t="n">
-        <v>2.24</v>
+        <v>2.05</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -1298,7 +1298,7 @@
         <v>6</v>
       </c>
       <c r="C50" t="n">
-        <v>-3.38</v>
+        <v>-3.3</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -1315,7 +1315,7 @@
         <v>8</v>
       </c>
       <c r="C51" t="n">
-        <v>-1.61</v>
+        <v>-1.53</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         <v>9</v>
       </c>
       <c r="C52" t="n">
-        <v>4.69</v>
+        <v>4.79</v>
       </c>
       <c r="D52" t="n">
         <v>1</v>
@@ -1349,7 +1349,7 @@
         <v>10</v>
       </c>
       <c r="C53" t="n">
-        <v>-0.77</v>
+        <v>-1.1</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>11</v>
       </c>
       <c r="C54" t="n">
-        <v>2.11</v>
+        <v>2.05</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -1383,7 +1383,7 @@
         <v>12</v>
       </c>
       <c r="C55" t="n">
-        <v>-1.03</v>
+        <v>-0.9</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>6</v>
       </c>
       <c r="C56" t="n">
-        <v>6.98</v>
+        <v>6.92</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
@@ -1417,7 +1417,7 @@
         <v>8</v>
       </c>
       <c r="C57" t="n">
-        <v>-6.5</v>
+        <v>-5.69</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -1434,7 +1434,7 @@
         <v>9</v>
       </c>
       <c r="C58" t="n">
-        <v>1.01</v>
+        <v>0.91</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1451,7 +1451,7 @@
         <v>10</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.58</v>
+        <v>-2.12</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>11</v>
       </c>
       <c r="C60" t="n">
-        <v>3.63</v>
+        <v>3.87</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>12</v>
       </c>
       <c r="C61" t="n">
-        <v>-4.55</v>
+        <v>-3.89</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1502,7 +1502,7 @@
         <v>6</v>
       </c>
       <c r="C62" t="n">
-        <v>1.97</v>
+        <v>2.08</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -1519,7 +1519,7 @@
         <v>8</v>
       </c>
       <c r="C63" t="n">
-        <v>2.74</v>
+        <v>2.79</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -1536,7 +1536,7 @@
         <v>9</v>
       </c>
       <c r="C64" t="n">
-        <v>0.54</v>
+        <v>0.62</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
         <v>10</v>
       </c>
       <c r="C65" t="n">
-        <v>-14.23</v>
+        <v>-14.37</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -1570,7 +1570,7 @@
         <v>11</v>
       </c>
       <c r="C66" t="n">
-        <v>4.05</v>
+        <v>3.96</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -1587,7 +1587,7 @@
         <v>12</v>
       </c>
       <c r="C67" t="n">
-        <v>4.93</v>
+        <v>4.92</v>
       </c>
       <c r="D67" t="n">
         <v>1</v>
@@ -1604,7 +1604,7 @@
         <v>6</v>
       </c>
       <c r="C68" t="n">
-        <v>-8.1</v>
+        <v>-8.44</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -1621,7 +1621,7 @@
         <v>8</v>
       </c>
       <c r="C69" t="n">
-        <v>-0.79</v>
+        <v>-1.25</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -1638,7 +1638,7 @@
         <v>9</v>
       </c>
       <c r="C70" t="n">
-        <v>5.58</v>
+        <v>5.29</v>
       </c>
       <c r="D70" t="n">
         <v>1</v>
@@ -1655,7 +1655,7 @@
         <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>-2.18</v>
+        <v>0.19</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
@@ -1672,7 +1672,7 @@
         <v>11</v>
       </c>
       <c r="C72" t="n">
-        <v>2.73</v>
+        <v>2.31</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -1689,7 +1689,7 @@
         <v>12</v>
       </c>
       <c r="C73" t="n">
-        <v>2.76</v>
+        <v>1.92</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>6</v>
       </c>
       <c r="C74" t="n">
-        <v>-1.64</v>
+        <v>-1.81</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -1723,7 +1723,7 @@
         <v>8</v>
       </c>
       <c r="C75" t="n">
-        <v>5.34</v>
+        <v>5.12</v>
       </c>
       <c r="D75" t="n">
         <v>1</v>
@@ -1740,7 +1740,7 @@
         <v>9</v>
       </c>
       <c r="C76" t="n">
-        <v>2.42</v>
+        <v>3.48</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -1757,7 +1757,7 @@
         <v>10</v>
       </c>
       <c r="C77" t="n">
-        <v>-8.47</v>
+        <v>-9.57</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -1774,7 +1774,7 @@
         <v>11</v>
       </c>
       <c r="C78" t="n">
-        <v>-1.67</v>
+        <v>-1.24</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -1808,7 +1808,7 @@
         <v>6</v>
       </c>
       <c r="C80" t="n">
-        <v>-5.66</v>
+        <v>-4.77</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>8</v>
       </c>
       <c r="C81" t="n">
-        <v>2.65</v>
+        <v>3.23</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -1842,7 +1842,7 @@
         <v>9</v>
       </c>
       <c r="C82" t="n">
-        <v>3.73</v>
+        <v>3.82</v>
       </c>
       <c r="D82" t="n">
         <v>1</v>
@@ -1859,7 +1859,7 @@
         <v>10</v>
       </c>
       <c r="C83" t="n">
-        <v>-6.29</v>
+        <v>-7.83</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -1876,7 +1876,7 @@
         <v>11</v>
       </c>
       <c r="C84" t="n">
-        <v>2.69</v>
+        <v>2.53</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -1893,7 +1893,7 @@
         <v>12</v>
       </c>
       <c r="C85" t="n">
-        <v>2.87</v>
+        <v>3.01</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -1910,7 +1910,7 @@
         <v>6</v>
       </c>
       <c r="C86" t="n">
-        <v>-1</v>
+        <v>-1.02</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>8</v>
       </c>
       <c r="C87" t="n">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="D87" t="n">
         <v>0</v>
@@ -1944,7 +1944,7 @@
         <v>9</v>
       </c>
       <c r="C88" t="n">
-        <v>3.27</v>
+        <v>3.26</v>
       </c>
       <c r="D88" t="n">
         <v>1</v>
@@ -1961,7 +1961,7 @@
         <v>10</v>
       </c>
       <c r="C89" t="n">
-        <v>-6.56</v>
+        <v>-8.25</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -1978,7 +1978,7 @@
         <v>11</v>
       </c>
       <c r="C90" t="n">
-        <v>1.71</v>
+        <v>3.15</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -1995,7 +1995,7 @@
         <v>12</v>
       </c>
       <c r="C91" t="n">
-        <v>1.02</v>
+        <v>1.32</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
@@ -2012,7 +2012,7 @@
         <v>6</v>
       </c>
       <c r="C92" t="n">
-        <v>10.05</v>
+        <v>10.3</v>
       </c>
       <c r="D92" t="n">
         <v>1</v>
@@ -2029,7 +2029,7 @@
         <v>8</v>
       </c>
       <c r="C93" t="n">
-        <v>6.36</v>
+        <v>6.27</v>
       </c>
       <c r="D93" t="n">
         <v>0</v>
@@ -2046,7 +2046,7 @@
         <v>9</v>
       </c>
       <c r="C94" t="n">
-        <v>0.64</v>
+        <v>0.48</v>
       </c>
       <c r="D94" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
         <v>10</v>
       </c>
       <c r="C95" t="n">
-        <v>-12.36</v>
+        <v>-12.09</v>
       </c>
       <c r="D95" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>11</v>
       </c>
       <c r="C96" t="n">
-        <v>-7.39</v>
+        <v>-7.63</v>
       </c>
       <c r="D96" t="n">
         <v>0</v>
@@ -2097,7 +2097,7 @@
         <v>12</v>
       </c>
       <c r="C97" t="n">
-        <v>2.71</v>
+        <v>2.66</v>
       </c>
       <c r="D97" t="n">
         <v>0</v>
@@ -2114,7 +2114,7 @@
         <v>6</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.87</v>
+        <v>-0.83</v>
       </c>
       <c r="D98" t="n">
         <v>0</v>
@@ -2131,7 +2131,7 @@
         <v>8</v>
       </c>
       <c r="C99" t="n">
-        <v>0.1</v>
+        <v>0.37</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>9</v>
       </c>
       <c r="C100" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="D100" t="n">
         <v>0</v>
@@ -2165,7 +2165,7 @@
         <v>10</v>
       </c>
       <c r="C101" t="n">
-        <v>-7.38</v>
+        <v>-6.9</v>
       </c>
       <c r="D101" t="n">
         <v>0</v>
@@ -2182,7 +2182,7 @@
         <v>11</v>
       </c>
       <c r="C102" t="n">
-        <v>3.79</v>
+        <v>3.66</v>
       </c>
       <c r="D102" t="n">
         <v>1</v>
@@ -2199,7 +2199,7 @@
         <v>12</v>
       </c>
       <c r="C103" t="n">
-        <v>1.96</v>
+        <v>1.99</v>
       </c>
       <c r="D103" t="n">
         <v>0</v>
@@ -2216,7 +2216,7 @@
         <v>6</v>
       </c>
       <c r="C104" t="n">
-        <v>-14.65</v>
+        <v>-14.45</v>
       </c>
       <c r="D104" t="n">
         <v>0</v>
@@ -2233,7 +2233,7 @@
         <v>8</v>
       </c>
       <c r="C105" t="n">
-        <v>2.39</v>
+        <v>2.37</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -2250,7 +2250,7 @@
         <v>9</v>
       </c>
       <c r="C106" t="n">
-        <v>2.8</v>
+        <v>3.25</v>
       </c>
       <c r="D106" t="n">
         <v>0</v>
@@ -2267,7 +2267,7 @@
         <v>10</v>
       </c>
       <c r="C107" t="n">
-        <v>2.03</v>
+        <v>0.39</v>
       </c>
       <c r="D107" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>11</v>
       </c>
       <c r="C108" t="n">
-        <v>0.83</v>
+        <v>1.2</v>
       </c>
       <c r="D108" t="n">
         <v>0</v>
@@ -2301,7 +2301,7 @@
         <v>12</v>
       </c>
       <c r="C109" t="n">
-        <v>6.6</v>
+        <v>7.24</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -2318,7 +2318,7 @@
         <v>6</v>
       </c>
       <c r="C110" t="n">
-        <v>-1.83</v>
+        <v>-1.8</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>8</v>
       </c>
       <c r="C111" t="n">
-        <v>1.06</v>
+        <v>0.75</v>
       </c>
       <c r="D111" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>9</v>
       </c>
       <c r="C112" t="n">
-        <v>1.79</v>
+        <v>2.29</v>
       </c>
       <c r="D112" t="n">
         <v>0</v>
@@ -2369,7 +2369,7 @@
         <v>10</v>
       </c>
       <c r="C113" t="n">
-        <v>-7</v>
+        <v>-6.72</v>
       </c>
       <c r="D113" t="n">
         <v>0</v>
@@ -2386,7 +2386,7 @@
         <v>11</v>
       </c>
       <c r="C114" t="n">
-        <v>0.87</v>
+        <v>0.5</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
@@ -2403,7 +2403,7 @@
         <v>12</v>
       </c>
       <c r="C115" t="n">
-        <v>5.12</v>
+        <v>4.99</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -2420,7 +2420,7 @@
         <v>6</v>
       </c>
       <c r="C116" t="n">
-        <v>-2.64</v>
+        <v>-2.61</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -2437,7 +2437,7 @@
         <v>8</v>
       </c>
       <c r="C117" t="n">
-        <v>2.65</v>
+        <v>2.76</v>
       </c>
       <c r="D117" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v>9</v>
       </c>
       <c r="C118" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="D118" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>10</v>
       </c>
       <c r="C119" t="n">
-        <v>-12.32</v>
+        <v>-12.33</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
@@ -2488,7 +2488,7 @@
         <v>11</v>
       </c>
       <c r="C120" t="n">
-        <v>2.28</v>
+        <v>2.29</v>
       </c>
       <c r="D120" t="n">
         <v>0</v>
@@ -2505,7 +2505,7 @@
         <v>12</v>
       </c>
       <c r="C121" t="n">
-        <v>8.06</v>
+        <v>7.9</v>
       </c>
       <c r="D121" t="n">
         <v>1</v>
@@ -2522,7 +2522,7 @@
         <v>6</v>
       </c>
       <c r="C122" t="n">
-        <v>-10.38</v>
+        <v>-10.6</v>
       </c>
       <c r="D122" t="n">
         <v>0</v>
@@ -2539,7 +2539,7 @@
         <v>8</v>
       </c>
       <c r="C123" t="n">
-        <v>6.77</v>
+        <v>6.97</v>
       </c>
       <c r="D123" t="n">
         <v>1</v>
@@ -2556,7 +2556,7 @@
         <v>9</v>
       </c>
       <c r="C124" t="n">
-        <v>4.99</v>
+        <v>4.34</v>
       </c>
       <c r="D124" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
         <v>10</v>
       </c>
       <c r="C125" t="n">
-        <v>-4.95</v>
+        <v>-4.46</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -2590,7 +2590,7 @@
         <v>11</v>
       </c>
       <c r="C126" t="n">
-        <v>0.65</v>
+        <v>0.67</v>
       </c>
       <c r="D126" t="n">
         <v>0</v>
@@ -2607,7 +2607,7 @@
         <v>12</v>
       </c>
       <c r="C127" t="n">
-        <v>2.92</v>
+        <v>3.08</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>6</v>
       </c>
       <c r="C128" t="n">
-        <v>-12.9</v>
+        <v>-12.85</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>-3.53</v>
+        <v>-3.76</v>
       </c>
       <c r="D129" t="n">
         <v>0</v>
@@ -2658,7 +2658,7 @@
         <v>9</v>
       </c>
       <c r="C130" t="n">
-        <v>4.86</v>
+        <v>4.21</v>
       </c>
       <c r="D130" t="n">
         <v>0</v>
@@ -2675,7 +2675,7 @@
         <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>10.53</v>
+        <v>10.81</v>
       </c>
       <c r="D131" t="n">
         <v>1</v>
@@ -2692,7 +2692,7 @@
         <v>11</v>
       </c>
       <c r="C132" t="n">
-        <v>4.69</v>
+        <v>5.06</v>
       </c>
       <c r="D132" t="n">
         <v>0</v>
@@ -2709,7 +2709,7 @@
         <v>12</v>
       </c>
       <c r="C133" t="n">
-        <v>-3.65</v>
+        <v>-3.47</v>
       </c>
       <c r="D133" t="n">
         <v>0</v>
@@ -2726,7 +2726,7 @@
         <v>6</v>
       </c>
       <c r="C134" t="n">
-        <v>-13.2</v>
+        <v>-13.37</v>
       </c>
       <c r="D134" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
         <v>8</v>
       </c>
       <c r="C135" t="n">
-        <v>5.86</v>
+        <v>5.9</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -2760,7 +2760,7 @@
         <v>9</v>
       </c>
       <c r="C136" t="n">
-        <v>3.15</v>
+        <v>3.05</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -2777,7 +2777,7 @@
         <v>10</v>
       </c>
       <c r="C137" t="n">
-        <v>-6.55</v>
+        <v>-6.39</v>
       </c>
       <c r="D137" t="n">
         <v>0</v>
@@ -2794,7 +2794,7 @@
         <v>11</v>
       </c>
       <c r="C138" t="n">
-        <v>6.5</v>
+        <v>6.54</v>
       </c>
       <c r="D138" t="n">
         <v>1</v>
@@ -2811,7 +2811,7 @@
         <v>12</v>
       </c>
       <c r="C139" t="n">
-        <v>4.24</v>
+        <v>4.27</v>
       </c>
       <c r="D139" t="n">
         <v>0</v>
@@ -2828,7 +2828,7 @@
         <v>6</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.47</v>
+        <v>-0.27</v>
       </c>
       <c r="D140" t="n">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>8</v>
       </c>
       <c r="C141" t="n">
-        <v>-4.44</v>
+        <v>-3.9</v>
       </c>
       <c r="D141" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>9</v>
       </c>
       <c r="C142" t="n">
-        <v>2.14</v>
+        <v>2.19</v>
       </c>
       <c r="D142" t="n">
         <v>0</v>
@@ -2879,7 +2879,7 @@
         <v>10</v>
       </c>
       <c r="C143" t="n">
-        <v>-6.73</v>
+        <v>-7.23</v>
       </c>
       <c r="D143" t="n">
         <v>0</v>
@@ -2896,7 +2896,7 @@
         <v>11</v>
       </c>
       <c r="C144" t="n">
-        <v>-0.35</v>
+        <v>-0.6</v>
       </c>
       <c r="D144" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>12</v>
       </c>
       <c r="C145" t="n">
-        <v>9.85</v>
+        <v>9.8</v>
       </c>
       <c r="D145" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Update Chancroid forecast data and related outputs
Refreshed Chancroid.csv with updated forecast values and intervals. This update likely reflects new model runs or corrections, and ensures consistency with other updated outputs and figures in the repository.
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Best_model_outcome.xlsx
+++ b/Outcome/Appendix/Best_model_outcome.xlsx
@@ -482,7 +482,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>2.9</v>
+        <v>2.79</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -499,7 +499,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>7.44</v>
+        <v>7.31</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -516,7 +516,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>-1.3</v>
+        <v>-0.7</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -533,7 +533,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>-11.78</v>
+        <v>-11.88</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -550,7 +550,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>-2.79</v>
+        <v>-2.94</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -567,7 +567,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>5.53</v>
+        <v>5.41</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -584,7 +584,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.61</v>
+        <v>-0.73</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -601,7 +601,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -618,7 +618,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>1.92</v>
+        <v>2.08</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -635,7 +635,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.63</v>
+        <v>0.69</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.82</v>
+        <v>-0.75</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -669,7 +669,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>-2.31</v>
+        <v>-2.48</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -686,7 +686,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>-4.02</v>
+        <v>-3.99</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -703,7 +703,7 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>3.07</v>
+        <v>3.1</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -720,7 +720,7 @@
         <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>3.99</v>
+        <v>3.91</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -771,7 +771,7 @@
         <v>12</v>
       </c>
       <c r="C19" t="n">
-        <v>1.75</v>
+        <v>1.77</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>9.16</v>
+        <v>9.17</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
@@ -805,7 +805,7 @@
         <v>8</v>
       </c>
       <c r="C21" t="n">
-        <v>-2.57</v>
+        <v>-2.56</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -822,7 +822,7 @@
         <v>9</v>
       </c>
       <c r="C22" t="n">
-        <v>-1.1</v>
+        <v>-1.13</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -839,7 +839,7 @@
         <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>2.93</v>
+        <v>2.94</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -873,7 +873,7 @@
         <v>12</v>
       </c>
       <c r="C25" t="n">
-        <v>3.67</v>
+        <v>3.68</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -890,7 +890,7 @@
         <v>6</v>
       </c>
       <c r="C26" t="n">
-        <v>2.29</v>
+        <v>2.31</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -907,7 +907,7 @@
         <v>8</v>
       </c>
       <c r="C27" t="n">
-        <v>2.92</v>
+        <v>2.91</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -924,7 +924,7 @@
         <v>9</v>
       </c>
       <c r="C28" t="n">
-        <v>4.85</v>
+        <v>4.84</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
@@ -958,7 +958,7 @@
         <v>11</v>
       </c>
       <c r="C30" t="n">
-        <v>0.07</v>
+        <v>0.1</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
         <v>12</v>
       </c>
       <c r="C31" t="n">
-        <v>1.64</v>
+        <v>1.62</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -992,7 +992,7 @@
         <v>6</v>
       </c>
       <c r="C32" t="n">
-        <v>8.35</v>
+        <v>8.41</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
@@ -1009,7 +1009,7 @@
         <v>8</v>
       </c>
       <c r="C33" t="n">
-        <v>1.47</v>
+        <v>1.58</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1026,7 +1026,7 @@
         <v>9</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.07</v>
+        <v>-0.69</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
         <v>10</v>
       </c>
       <c r="C35" t="n">
-        <v>-14.08</v>
+        <v>-13.89</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1060,7 +1060,7 @@
         <v>11</v>
       </c>
       <c r="C36" t="n">
-        <v>4.06</v>
+        <v>4.22</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>12</v>
       </c>
       <c r="C37" t="n">
-        <v>0.27</v>
+        <v>0.37</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1094,7 +1094,7 @@
         <v>6</v>
       </c>
       <c r="C38" t="n">
-        <v>-6.06</v>
+        <v>-6.07</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -1111,7 +1111,7 @@
         <v>8</v>
       </c>
       <c r="C39" t="n">
-        <v>3.81</v>
+        <v>3.79</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1128,7 +1128,7 @@
         <v>9</v>
       </c>
       <c r="C40" t="n">
-        <v>4.03</v>
+        <v>4.13</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1145,7 +1145,7 @@
         <v>10</v>
       </c>
       <c r="C41" t="n">
-        <v>0.02</v>
+        <v>-0.01</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1162,7 +1162,7 @@
         <v>11</v>
       </c>
       <c r="C42" t="n">
-        <v>-8.79</v>
+        <v>-8.8</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -1179,7 +1179,7 @@
         <v>12</v>
       </c>
       <c r="C43" t="n">
-        <v>6.98</v>
+        <v>6.96</v>
       </c>
       <c r="D43" t="n">
         <v>1</v>
@@ -1213,7 +1213,7 @@
         <v>8</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.94</v>
+        <v>-0.95</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1247,7 +1247,7 @@
         <v>10</v>
       </c>
       <c r="C47" t="n">
-        <v>-5.9</v>
+        <v>-5.91</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
@@ -1298,7 +1298,7 @@
         <v>6</v>
       </c>
       <c r="C50" t="n">
-        <v>-3.3</v>
+        <v>-3.31</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -1315,7 +1315,7 @@
         <v>8</v>
       </c>
       <c r="C51" t="n">
-        <v>-1.53</v>
+        <v>-1.54</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         <v>9</v>
       </c>
       <c r="C52" t="n">
-        <v>4.79</v>
+        <v>4.84</v>
       </c>
       <c r="D52" t="n">
         <v>1</v>
@@ -1349,7 +1349,7 @@
         <v>10</v>
       </c>
       <c r="C53" t="n">
-        <v>-1.1</v>
+        <v>-1.12</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>11</v>
       </c>
       <c r="C54" t="n">
-        <v>2.05</v>
+        <v>2.03</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>6</v>
       </c>
       <c r="C56" t="n">
-        <v>6.92</v>
+        <v>6.94</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
@@ -1417,7 +1417,7 @@
         <v>8</v>
       </c>
       <c r="C57" t="n">
-        <v>-5.69</v>
+        <v>-5.7</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -1434,7 +1434,7 @@
         <v>9</v>
       </c>
       <c r="C58" t="n">
-        <v>0.91</v>
+        <v>0.86</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1451,7 +1451,7 @@
         <v>10</v>
       </c>
       <c r="C59" t="n">
-        <v>-2.12</v>
+        <v>-2.13</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>11</v>
       </c>
       <c r="C60" t="n">
-        <v>3.87</v>
+        <v>3.94</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>12</v>
       </c>
       <c r="C61" t="n">
-        <v>-3.89</v>
+        <v>-3.9</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1519,7 +1519,7 @@
         <v>8</v>
       </c>
       <c r="C63" t="n">
-        <v>2.79</v>
+        <v>2.8</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -1536,7 +1536,7 @@
         <v>9</v>
       </c>
       <c r="C64" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
         <v>10</v>
       </c>
       <c r="C65" t="n">
-        <v>-14.37</v>
+        <v>-14.36</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -1587,7 +1587,7 @@
         <v>12</v>
       </c>
       <c r="C67" t="n">
-        <v>4.92</v>
+        <v>4.93</v>
       </c>
       <c r="D67" t="n">
         <v>1</v>
@@ -1638,7 +1638,7 @@
         <v>9</v>
       </c>
       <c r="C70" t="n">
-        <v>5.29</v>
+        <v>5.23</v>
       </c>
       <c r="D70" t="n">
         <v>1</v>
@@ -1655,7 +1655,7 @@
         <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
@@ -1672,7 +1672,7 @@
         <v>11</v>
       </c>
       <c r="C72" t="n">
-        <v>2.31</v>
+        <v>2.32</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -1689,7 +1689,7 @@
         <v>12</v>
       </c>
       <c r="C73" t="n">
-        <v>1.92</v>
+        <v>1.93</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>6</v>
       </c>
       <c r="C74" t="n">
-        <v>-1.81</v>
+        <v>-1.82</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -1723,7 +1723,7 @@
         <v>8</v>
       </c>
       <c r="C75" t="n">
-        <v>5.12</v>
+        <v>5.11</v>
       </c>
       <c r="D75" t="n">
         <v>1</v>
@@ -1740,7 +1740,7 @@
         <v>9</v>
       </c>
       <c r="C76" t="n">
-        <v>3.48</v>
+        <v>3.52</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -1774,7 +1774,7 @@
         <v>11</v>
       </c>
       <c r="C78" t="n">
-        <v>-1.24</v>
+        <v>-1.25</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -1791,7 +1791,7 @@
         <v>12</v>
       </c>
       <c r="C79" t="n">
-        <v>4.02</v>
+        <v>4.01</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -1808,7 +1808,7 @@
         <v>6</v>
       </c>
       <c r="C80" t="n">
-        <v>-4.77</v>
+        <v>-4.76</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>8</v>
       </c>
       <c r="C81" t="n">
-        <v>3.23</v>
+        <v>3.22</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -1842,7 +1842,7 @@
         <v>9</v>
       </c>
       <c r="C82" t="n">
-        <v>3.82</v>
+        <v>3.88</v>
       </c>
       <c r="D82" t="n">
         <v>1</v>
@@ -1859,7 +1859,7 @@
         <v>10</v>
       </c>
       <c r="C83" t="n">
-        <v>-7.83</v>
+        <v>-7.86</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -1876,7 +1876,7 @@
         <v>11</v>
       </c>
       <c r="C84" t="n">
-        <v>2.53</v>
+        <v>2.52</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -1893,7 +1893,7 @@
         <v>12</v>
       </c>
       <c r="C85" t="n">
-        <v>3.01</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -2046,7 +2046,7 @@
         <v>9</v>
       </c>
       <c r="C94" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="D94" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>11</v>
       </c>
       <c r="C96" t="n">
-        <v>-7.63</v>
+        <v>-7.62</v>
       </c>
       <c r="D96" t="n">
         <v>0</v>
@@ -2114,7 +2114,7 @@
         <v>6</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.83</v>
+        <v>-0.8</v>
       </c>
       <c r="D98" t="n">
         <v>0</v>
@@ -2131,7 +2131,7 @@
         <v>8</v>
       </c>
       <c r="C99" t="n">
-        <v>0.37</v>
+        <v>0.43</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>9</v>
       </c>
       <c r="C100" t="n">
-        <v>1.7</v>
+        <v>1.66</v>
       </c>
       <c r="D100" t="n">
         <v>0</v>
@@ -2165,7 +2165,7 @@
         <v>10</v>
       </c>
       <c r="C101" t="n">
-        <v>-6.9</v>
+        <v>-6.95</v>
       </c>
       <c r="D101" t="n">
         <v>0</v>
@@ -2182,7 +2182,7 @@
         <v>11</v>
       </c>
       <c r="C102" t="n">
-        <v>3.66</v>
+        <v>3.63</v>
       </c>
       <c r="D102" t="n">
         <v>1</v>
@@ -2199,7 +2199,7 @@
         <v>12</v>
       </c>
       <c r="C103" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="D103" t="n">
         <v>0</v>
@@ -2233,7 +2233,7 @@
         <v>8</v>
       </c>
       <c r="C105" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -2250,7 +2250,7 @@
         <v>9</v>
       </c>
       <c r="C106" t="n">
-        <v>3.25</v>
+        <v>3.31</v>
       </c>
       <c r="D106" t="n">
         <v>0</v>
@@ -2267,7 +2267,7 @@
         <v>10</v>
       </c>
       <c r="C107" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="D107" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>11</v>
       </c>
       <c r="C108" t="n">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="D108" t="n">
         <v>0</v>
@@ -2301,7 +2301,7 @@
         <v>12</v>
       </c>
       <c r="C109" t="n">
-        <v>7.24</v>
+        <v>7.23</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -2318,7 +2318,7 @@
         <v>6</v>
       </c>
       <c r="C110" t="n">
-        <v>-1.8</v>
+        <v>-1.79</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>8</v>
       </c>
       <c r="C111" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="D111" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>9</v>
       </c>
       <c r="C112" t="n">
-        <v>2.29</v>
+        <v>2.21</v>
       </c>
       <c r="D112" t="n">
         <v>0</v>
@@ -2369,7 +2369,7 @@
         <v>10</v>
       </c>
       <c r="C113" t="n">
-        <v>-6.72</v>
+        <v>-6.7</v>
       </c>
       <c r="D113" t="n">
         <v>0</v>
@@ -2386,7 +2386,7 @@
         <v>11</v>
       </c>
       <c r="C114" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
@@ -2403,7 +2403,7 @@
         <v>12</v>
       </c>
       <c r="C115" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -2420,7 +2420,7 @@
         <v>6</v>
       </c>
       <c r="C116" t="n">
-        <v>-2.61</v>
+        <v>-2.64</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -2437,7 +2437,7 @@
         <v>8</v>
       </c>
       <c r="C117" t="n">
-        <v>2.76</v>
+        <v>2.73</v>
       </c>
       <c r="D117" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v>9</v>
       </c>
       <c r="C118" t="n">
-        <v>2</v>
+        <v>2.15</v>
       </c>
       <c r="D118" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>10</v>
       </c>
       <c r="C119" t="n">
-        <v>-12.33</v>
+        <v>-12.38</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
@@ -2488,7 +2488,7 @@
         <v>11</v>
       </c>
       <c r="C120" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="D120" t="n">
         <v>0</v>
@@ -2505,7 +2505,7 @@
         <v>12</v>
       </c>
       <c r="C121" t="n">
-        <v>7.9</v>
+        <v>7.87</v>
       </c>
       <c r="D121" t="n">
         <v>1</v>
@@ -2522,7 +2522,7 @@
         <v>6</v>
       </c>
       <c r="C122" t="n">
-        <v>-10.6</v>
+        <v>-10.61</v>
       </c>
       <c r="D122" t="n">
         <v>0</v>
@@ -2539,7 +2539,7 @@
         <v>8</v>
       </c>
       <c r="C123" t="n">
-        <v>6.97</v>
+        <v>6.89</v>
       </c>
       <c r="D123" t="n">
         <v>1</v>
@@ -2556,7 +2556,7 @@
         <v>9</v>
       </c>
       <c r="C124" t="n">
-        <v>4.34</v>
+        <v>4.56</v>
       </c>
       <c r="D124" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
         <v>10</v>
       </c>
       <c r="C125" t="n">
-        <v>-4.46</v>
+        <v>-4.52</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -2590,7 +2590,7 @@
         <v>11</v>
       </c>
       <c r="C126" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="D126" t="n">
         <v>0</v>
@@ -2607,7 +2607,7 @@
         <v>12</v>
       </c>
       <c r="C127" t="n">
-        <v>3.08</v>
+        <v>3.02</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>6</v>
       </c>
       <c r="C128" t="n">
-        <v>-12.85</v>
+        <v>-12.82</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>-3.76</v>
+        <v>-3.77</v>
       </c>
       <c r="D129" t="n">
         <v>0</v>
@@ -2658,7 +2658,7 @@
         <v>9</v>
       </c>
       <c r="C130" t="n">
-        <v>4.21</v>
+        <v>4.24</v>
       </c>
       <c r="D130" t="n">
         <v>0</v>
@@ -2675,7 +2675,7 @@
         <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>10.81</v>
+        <v>10.78</v>
       </c>
       <c r="D131" t="n">
         <v>1</v>
@@ -2692,7 +2692,7 @@
         <v>11</v>
       </c>
       <c r="C132" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="D132" t="n">
         <v>0</v>
@@ -2709,7 +2709,7 @@
         <v>12</v>
       </c>
       <c r="C133" t="n">
-        <v>-3.47</v>
+        <v>-3.48</v>
       </c>
       <c r="D133" t="n">
         <v>0</v>
@@ -2726,7 +2726,7 @@
         <v>6</v>
       </c>
       <c r="C134" t="n">
-        <v>-13.37</v>
+        <v>-13.36</v>
       </c>
       <c r="D134" t="n">
         <v>0</v>
@@ -2760,7 +2760,7 @@
         <v>9</v>
       </c>
       <c r="C136" t="n">
-        <v>3.05</v>
+        <v>3.03</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -2811,7 +2811,7 @@
         <v>12</v>
       </c>
       <c r="C139" t="n">
-        <v>4.27</v>
+        <v>4.28</v>
       </c>
       <c r="D139" t="n">
         <v>0</v>
@@ -2828,7 +2828,7 @@
         <v>6</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.27</v>
+        <v>-0.25</v>
       </c>
       <c r="D140" t="n">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>8</v>
       </c>
       <c r="C141" t="n">
-        <v>-3.9</v>
+        <v>-3.88</v>
       </c>
       <c r="D141" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>9</v>
       </c>
       <c r="C142" t="n">
-        <v>2.19</v>
+        <v>2.12</v>
       </c>
       <c r="D142" t="n">
         <v>0</v>
@@ -2879,7 +2879,7 @@
         <v>10</v>
       </c>
       <c r="C143" t="n">
-        <v>-7.23</v>
+        <v>-7.22</v>
       </c>
       <c r="D143" t="n">
         <v>0</v>
@@ -2896,7 +2896,7 @@
         <v>11</v>
       </c>
       <c r="C144" t="n">
-        <v>-0.6</v>
+        <v>-0.58</v>
       </c>
       <c r="D144" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>12</v>
       </c>
       <c r="C145" t="n">
-        <v>9.8</v>
+        <v>9.82</v>
       </c>
       <c r="D145" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Update forecast and outcome data for appendices
Refreshed forecast CSVs and Excel files in Outcome/Appendix with updated values for disease projections and model outcomes. Also updated population data and related figure files to reflect the latest analysis results.
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Best_model_outcome.xlsx
+++ b/Outcome/Appendix/Best_model_outcome.xlsx
@@ -482,7 +482,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>2.82</v>
+        <v>2.76</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -499,7 +499,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>7.36</v>
+        <v>7.28</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -516,7 +516,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.85</v>
+        <v>-0.43</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -533,7 +533,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>-11.86</v>
+        <v>-11.97</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -550,7 +550,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>-2.91</v>
+        <v>-3.01</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -567,7 +567,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>5.44</v>
+        <v>5.37</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -584,7 +584,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.62</v>
+        <v>-0.64</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -601,7 +601,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -618,7 +618,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>1.97</v>
+        <v>2.02</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -635,7 +635,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.83</v>
+        <v>-0.85</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -669,7 +669,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>-2.32</v>
+        <v>-2.33</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -686,7 +686,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>-4.03</v>
+        <v>-4.02</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -703,7 +703,7 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>3.06</v>
+        <v>3.07</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -720,7 +720,7 @@
         <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>4.04</v>
+        <v>4.03</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -737,7 +737,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>-4.79</v>
+        <v>-4.8</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -754,7 +754,7 @@
         <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>9.16</v>
+        <v>9.17</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
@@ -805,7 +805,7 @@
         <v>8</v>
       </c>
       <c r="C21" t="n">
-        <v>-2.58</v>
+        <v>-2.56</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -822,7 +822,7 @@
         <v>9</v>
       </c>
       <c r="C22" t="n">
-        <v>-1.08</v>
+        <v>-1.13</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -839,7 +839,7 @@
         <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>2.93</v>
+        <v>2.94</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -873,7 +873,7 @@
         <v>12</v>
       </c>
       <c r="C25" t="n">
-        <v>3.67</v>
+        <v>3.68</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -890,7 +890,7 @@
         <v>6</v>
       </c>
       <c r="C26" t="n">
-        <v>2.4</v>
+        <v>2.29</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -907,7 +907,7 @@
         <v>8</v>
       </c>
       <c r="C27" t="n">
-        <v>3.01</v>
+        <v>2.93</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -924,7 +924,7 @@
         <v>9</v>
       </c>
       <c r="C28" t="n">
-        <v>4.43</v>
+        <v>4.84</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
@@ -941,7 +941,7 @@
         <v>10</v>
       </c>
       <c r="C29" t="n">
-        <v>-11.74</v>
+        <v>-11.77</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -958,7 +958,7 @@
         <v>11</v>
       </c>
       <c r="C30" t="n">
-        <v>0.18</v>
+        <v>0.07</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
         <v>12</v>
       </c>
       <c r="C31" t="n">
-        <v>1.72</v>
+        <v>1.65</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -992,7 +992,7 @@
         <v>6</v>
       </c>
       <c r="C32" t="n">
-        <v>8.38</v>
+        <v>8.42</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
@@ -1009,7 +1009,7 @@
         <v>8</v>
       </c>
       <c r="C33" t="n">
-        <v>1.52</v>
+        <v>1.61</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1026,7 +1026,7 @@
         <v>9</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.34</v>
+        <v>-0.88</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
         <v>10</v>
       </c>
       <c r="C35" t="n">
-        <v>-14</v>
+        <v>-13.8</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1060,7 +1060,7 @@
         <v>11</v>
       </c>
       <c r="C36" t="n">
-        <v>4.12</v>
+        <v>4.26</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>12</v>
       </c>
       <c r="C37" t="n">
-        <v>0.32</v>
+        <v>0.4</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1111,7 +1111,7 @@
         <v>8</v>
       </c>
       <c r="C39" t="n">
-        <v>3.77</v>
+        <v>3.8</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1128,7 +1128,7 @@
         <v>9</v>
       </c>
       <c r="C40" t="n">
-        <v>4.23</v>
+        <v>4.07</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1145,7 +1145,7 @@
         <v>10</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.06</v>
+        <v>0.01</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1162,7 +1162,7 @@
         <v>11</v>
       </c>
       <c r="C42" t="n">
-        <v>-8.8</v>
+        <v>-8.79</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -1179,7 +1179,7 @@
         <v>12</v>
       </c>
       <c r="C43" t="n">
-        <v>6.92</v>
+        <v>6.97</v>
       </c>
       <c r="D43" t="n">
         <v>1</v>
@@ -1230,7 +1230,7 @@
         <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>9.04</v>
+        <v>9.06</v>
       </c>
       <c r="D46" t="n">
         <v>1</v>
@@ -1247,7 +1247,7 @@
         <v>10</v>
       </c>
       <c r="C47" t="n">
-        <v>-5.89</v>
+        <v>-5.9</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         <v>9</v>
       </c>
       <c r="C52" t="n">
-        <v>4.83</v>
+        <v>4.81</v>
       </c>
       <c r="D52" t="n">
         <v>1</v>
@@ -1400,7 +1400,7 @@
         <v>6</v>
       </c>
       <c r="C56" t="n">
-        <v>6.93</v>
+        <v>6.92</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
@@ -1434,7 +1434,7 @@
         <v>9</v>
       </c>
       <c r="C58" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>11</v>
       </c>
       <c r="C60" t="n">
-        <v>3.92</v>
+        <v>3.9</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>12</v>
       </c>
       <c r="C61" t="n">
-        <v>-3.88</v>
+        <v>-3.89</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1502,7 +1502,7 @@
         <v>6</v>
       </c>
       <c r="C62" t="n">
-        <v>2.06</v>
+        <v>2.08</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -1519,7 +1519,7 @@
         <v>8</v>
       </c>
       <c r="C63" t="n">
-        <v>2.77</v>
+        <v>2.79</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -1536,7 +1536,7 @@
         <v>9</v>
       </c>
       <c r="C64" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
         <v>10</v>
       </c>
       <c r="C65" t="n">
-        <v>-14.38</v>
+        <v>-14.37</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -1570,7 +1570,7 @@
         <v>11</v>
       </c>
       <c r="C66" t="n">
-        <v>3.94</v>
+        <v>3.96</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -1587,7 +1587,7 @@
         <v>12</v>
       </c>
       <c r="C67" t="n">
-        <v>4.91</v>
+        <v>4.93</v>
       </c>
       <c r="D67" t="n">
         <v>1</v>
@@ -1604,7 +1604,7 @@
         <v>6</v>
       </c>
       <c r="C68" t="n">
-        <v>-8.43</v>
+        <v>-8.44</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -1723,7 +1723,7 @@
         <v>8</v>
       </c>
       <c r="C75" t="n">
-        <v>5.12</v>
+        <v>5.11</v>
       </c>
       <c r="D75" t="n">
         <v>1</v>
@@ -1740,7 +1740,7 @@
         <v>9</v>
       </c>
       <c r="C76" t="n">
-        <v>3.49</v>
+        <v>3.52</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -1757,7 +1757,7 @@
         <v>10</v>
       </c>
       <c r="C77" t="n">
-        <v>-9.56</v>
+        <v>-9.57</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -1808,7 +1808,7 @@
         <v>6</v>
       </c>
       <c r="C80" t="n">
-        <v>-4.75</v>
+        <v>-4.78</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>8</v>
       </c>
       <c r="C81" t="n">
-        <v>3.25</v>
+        <v>3.2</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -1842,7 +1842,7 @@
         <v>9</v>
       </c>
       <c r="C82" t="n">
-        <v>3.73</v>
+        <v>4.01</v>
       </c>
       <c r="D82" t="n">
         <v>1</v>
@@ -1859,7 +1859,7 @@
         <v>10</v>
       </c>
       <c r="C83" t="n">
-        <v>-7.81</v>
+        <v>-7.9</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -1876,7 +1876,7 @@
         <v>11</v>
       </c>
       <c r="C84" t="n">
-        <v>2.55</v>
+        <v>2.49</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -1893,7 +1893,7 @@
         <v>12</v>
       </c>
       <c r="C85" t="n">
-        <v>3.03</v>
+        <v>2.98</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>8</v>
       </c>
       <c r="C87" t="n">
-        <v>1.54</v>
+        <v>1.55</v>
       </c>
       <c r="D87" t="n">
         <v>0</v>
@@ -1944,7 +1944,7 @@
         <v>9</v>
       </c>
       <c r="C88" t="n">
-        <v>3.27</v>
+        <v>3.22</v>
       </c>
       <c r="D88" t="n">
         <v>1</v>
@@ -1961,7 +1961,7 @@
         <v>10</v>
       </c>
       <c r="C89" t="n">
-        <v>-8.26</v>
+        <v>-8.25</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -1995,7 +1995,7 @@
         <v>12</v>
       </c>
       <c r="C91" t="n">
-        <v>1.32</v>
+        <v>1.34</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
@@ -2046,7 +2046,7 @@
         <v>9</v>
       </c>
       <c r="C94" t="n">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="D94" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>11</v>
       </c>
       <c r="C96" t="n">
-        <v>-7.62</v>
+        <v>-7.63</v>
       </c>
       <c r="D96" t="n">
         <v>0</v>
@@ -2114,7 +2114,7 @@
         <v>6</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.79</v>
+        <v>-0.73</v>
       </c>
       <c r="D98" t="n">
         <v>0</v>
@@ -2131,7 +2131,7 @@
         <v>8</v>
       </c>
       <c r="C99" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>9</v>
       </c>
       <c r="C100" t="n">
-        <v>1.57</v>
+        <v>1.2</v>
       </c>
       <c r="D100" t="n">
         <v>0</v>
@@ -2165,7 +2165,7 @@
         <v>10</v>
       </c>
       <c r="C101" t="n">
-        <v>-6.91</v>
+        <v>-6.84</v>
       </c>
       <c r="D101" t="n">
         <v>0</v>
@@ -2182,7 +2182,7 @@
         <v>11</v>
       </c>
       <c r="C102" t="n">
-        <v>3.67</v>
+        <v>3.86</v>
       </c>
       <c r="D102" t="n">
         <v>1</v>
@@ -2199,7 +2199,7 @@
         <v>12</v>
       </c>
       <c r="C103" t="n">
-        <v>2.04</v>
+        <v>2.08</v>
       </c>
       <c r="D103" t="n">
         <v>0</v>
@@ -2216,7 +2216,7 @@
         <v>6</v>
       </c>
       <c r="C104" t="n">
-        <v>-14.48</v>
+        <v>-14.49</v>
       </c>
       <c r="D104" t="n">
         <v>0</v>
@@ -2233,7 +2233,7 @@
         <v>8</v>
       </c>
       <c r="C105" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -2250,7 +2250,7 @@
         <v>9</v>
       </c>
       <c r="C106" t="n">
-        <v>3.48</v>
+        <v>3.47</v>
       </c>
       <c r="D106" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>11</v>
       </c>
       <c r="C108" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="D108" t="n">
         <v>0</v>
@@ -2301,7 +2301,7 @@
         <v>12</v>
       </c>
       <c r="C109" t="n">
-        <v>7.19</v>
+        <v>7.2</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -2318,7 +2318,7 @@
         <v>6</v>
       </c>
       <c r="C110" t="n">
-        <v>-1.82</v>
+        <v>-1.81</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>8</v>
       </c>
       <c r="C111" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="D111" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>9</v>
       </c>
       <c r="C112" t="n">
-        <v>2.43</v>
+        <v>2.44</v>
       </c>
       <c r="D112" t="n">
         <v>0</v>
@@ -2369,7 +2369,7 @@
         <v>10</v>
       </c>
       <c r="C113" t="n">
-        <v>-6.76</v>
+        <v>-6.77</v>
       </c>
       <c r="D113" t="n">
         <v>0</v>
@@ -2386,7 +2386,7 @@
         <v>11</v>
       </c>
       <c r="C114" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v>9</v>
       </c>
       <c r="C118" t="n">
-        <v>2.13</v>
+        <v>2.15</v>
       </c>
       <c r="D118" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>10</v>
       </c>
       <c r="C119" t="n">
-        <v>-12.37</v>
+        <v>-12.38</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
@@ -2522,7 +2522,7 @@
         <v>6</v>
       </c>
       <c r="C122" t="n">
-        <v>-10.67</v>
+        <v>-10.64</v>
       </c>
       <c r="D122" t="n">
         <v>0</v>
@@ -2539,7 +2539,7 @@
         <v>8</v>
       </c>
       <c r="C123" t="n">
-        <v>6.71</v>
+        <v>6.79</v>
       </c>
       <c r="D123" t="n">
         <v>1</v>
@@ -2556,7 +2556,7 @@
         <v>9</v>
       </c>
       <c r="C124" t="n">
-        <v>5.12</v>
+        <v>4.84</v>
       </c>
       <c r="D124" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
         <v>10</v>
       </c>
       <c r="C125" t="n">
-        <v>-4.64</v>
+        <v>-4.59</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -2590,7 +2590,7 @@
         <v>11</v>
       </c>
       <c r="C126" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="D126" t="n">
         <v>0</v>
@@ -2607,7 +2607,7 @@
         <v>12</v>
       </c>
       <c r="C127" t="n">
-        <v>2.87</v>
+        <v>2.94</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>6</v>
       </c>
       <c r="C128" t="n">
-        <v>-12.8</v>
+        <v>-12.84</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>-3.81</v>
+        <v>-3.78</v>
       </c>
       <c r="D129" t="n">
         <v>0</v>
@@ -2658,7 +2658,7 @@
         <v>9</v>
       </c>
       <c r="C130" t="n">
-        <v>4.43</v>
+        <v>4.31</v>
       </c>
       <c r="D130" t="n">
         <v>0</v>
@@ -2675,7 +2675,7 @@
         <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>10.69</v>
+        <v>10.76</v>
       </c>
       <c r="D131" t="n">
         <v>1</v>
@@ -2692,7 +2692,7 @@
         <v>11</v>
       </c>
       <c r="C132" t="n">
-        <v>5</v>
+        <v>5.03</v>
       </c>
       <c r="D132" t="n">
         <v>0</v>
@@ -2709,7 +2709,7 @@
         <v>12</v>
       </c>
       <c r="C133" t="n">
-        <v>-3.51</v>
+        <v>-3.49</v>
       </c>
       <c r="D133" t="n">
         <v>0</v>
@@ -2726,7 +2726,7 @@
         <v>6</v>
       </c>
       <c r="C134" t="n">
-        <v>-13.33</v>
+        <v>-13.34</v>
       </c>
       <c r="D134" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
         <v>8</v>
       </c>
       <c r="C135" t="n">
-        <v>5.98</v>
+        <v>5.94</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -2760,7 +2760,7 @@
         <v>9</v>
       </c>
       <c r="C136" t="n">
-        <v>2.72</v>
+        <v>2.87</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -2777,7 +2777,7 @@
         <v>10</v>
       </c>
       <c r="C137" t="n">
-        <v>-6.34</v>
+        <v>-6.37</v>
       </c>
       <c r="D137" t="n">
         <v>0</v>
@@ -2794,7 +2794,7 @@
         <v>11</v>
       </c>
       <c r="C138" t="n">
-        <v>6.62</v>
+        <v>6.58</v>
       </c>
       <c r="D138" t="n">
         <v>1</v>
@@ -2811,7 +2811,7 @@
         <v>12</v>
       </c>
       <c r="C139" t="n">
-        <v>4.35</v>
+        <v>4.32</v>
       </c>
       <c r="D139" t="n">
         <v>0</v>
@@ -2828,7 +2828,7 @@
         <v>6</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.27</v>
+        <v>-0.26</v>
       </c>
       <c r="D140" t="n">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>8</v>
       </c>
       <c r="C141" t="n">
-        <v>-3.9</v>
+        <v>-3.89</v>
       </c>
       <c r="D141" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>9</v>
       </c>
       <c r="C142" t="n">
-        <v>2.19</v>
+        <v>2.14</v>
       </c>
       <c r="D142" t="n">
         <v>0</v>
@@ -2896,7 +2896,7 @@
         <v>11</v>
       </c>
       <c r="C144" t="n">
-        <v>-0.6</v>
+        <v>-0.59</v>
       </c>
       <c r="D144" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>12</v>
       </c>
       <c r="C145" t="n">
-        <v>9.8</v>
+        <v>9.81</v>
       </c>
       <c r="D145" t="n">
         <v>1</v>

</xml_diff>